<commit_message>
Drive the bundle-saving term from Spotify's disclosed MLC contingency series
- Collect the cumulative MLC liability figure from every 6-K and 20-F
  since Q2-24 (data/mlc_contingency.csv) and derive quarterly increments
- Gross bundle saving now comes from the filings (2024: 150, 2025: 208)
  instead of a 13-month run-rate; 2026E-27E are flagged placeholders
- Add Billboard's MLC-report analysis as an independent cross-check of
  the quarterly discount (within EUR 1.3M of the filing increment)
- Hand-back covers five direct deals (UMPG, Warner Chappell, Kobalt,
  Sony Music Publishing, BMG); restoration set to 75% with evidence
- MLC-loss switch now removes only the independents' share
- Write analysis/mlc-bridge.md documenting the series, the cross-check,
  the bridge to B and N, and what changed

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Bq554HW2LcX3ZmUaAuu9U
</commit_message>
<xml_diff>
--- a/data/SPOT_audiobooks_model.xlsx
+++ b/data/SPOT_audiobooks_model.xlsx
@@ -17,10 +17,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="0_);(0)"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
+    <numFmt numFmtId="167" formatCode="0_);(0)"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -86,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -94,12 +95,13 @@
     <xf numFmtId="37" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="37" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="3" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -108,20 +110,25 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="37" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="37" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="37" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="37" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -488,7 +495,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="78" customWidth="1" min="1" max="1"/>
@@ -1268,11 +1275,11 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Bundle mechanical-royalty reduction, 1 Mar 2024 to 31 Mar 2025 (13 months)</t>
+          <t>MLC contingency, cumulative 1 Mar 2024 to 30 Jun 2024</t>
         </is>
       </c>
       <c r="B29" s="3" t="n">
-        <v>205</v>
+        <v>46</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1281,7 +1288,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Mar24-Mar25</t>
+          <t>Q2-24</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1291,507 +1298,539 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Spotify 6-K Q1-25: 'additional royalties that would be due would be approximately €205 million, plus potentially penalties and interest'</t>
+          <t>6-K Q2-24: 'approximately €46 million, of which approximately €35 million relates to the three months ended June 30, 2024'</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Months in the disclosure period</t>
-        </is>
-      </c>
-      <c r="B30" s="7" t="n">
-        <v>13</v>
+          <t>of which the three months April to June 2024</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>35</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>months</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr"/>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Q2-24</t>
+        </is>
+      </c>
       <c r="E30" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>6-K Q2-24 (same sentence)</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>NMPA estimate of first-year publisher loss</t>
+          <t>MLC contingency, cumulative to 30 Sep 2024</t>
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>230</v>
+        <v>94</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>$M</t>
+          <t>€M</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2024-25</t>
+          <t>Q3-24</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>NMPA via Billboard</t>
+          <t>6-K Q3-24</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Mechanical royalties paid, Q4-23 (MLC reports)</t>
+          <t>MLC contingency, cumulative to 31 Dec 2024</t>
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>97.3</v>
+        <v>150</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>$M</t>
+          <t>€M</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Q4-23</t>
+          <t>Q4-24</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Billboard analysis</t>
+          <t>20-F FY24</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Mechanical royalties paid, Q4-25 (MLC reports; majors direct-licensed, so not comparable after 2025)</t>
+          <t>MLC contingency, cumulative to 31 Mar 2025</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
-        <v>53.3</v>
+        <v>205</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>$M</t>
+          <t>€M</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Q4-25</t>
+          <t>Q1-25</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Billboard analysis</t>
+          <t>6-K Q1-25</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Music share of bundle revenue under CRB allocation</t>
-        </is>
-      </c>
-      <c r="B34" s="6" t="n">
-        <v>0.52</v>
+          <t>MLC contingency, cumulative to 30 Jun 2025</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>256</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr"/>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Q2-25</t>
+        </is>
+      </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>NMPA / Billboard ('$5.70 of the bundle')</t>
+          <t>6-K Q2-25</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>UMPG share of US mechanicals</t>
-        </is>
-      </c>
-      <c r="B35" s="8" t="n">
-        <v>0.22</v>
+          <t>MLC contingency, cumulative to 30 Sep 2025</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>308</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr"/>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Q3-25</t>
+        </is>
+      </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Estimate from US publishing market shares (range 20-25%)</t>
+          <t>6-K Q3-25: first filing to add 'Any liability would be partially offset by direct deals with publishers'</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Warner Chappell share of US mechanicals</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="n">
-        <v>0.13</v>
+          <t>MLC contingency, cumulative to 31 Dec 2025</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>358</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr"/>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Q4-25</t>
+        </is>
+      </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Estimate (range 11-15%)</t>
+          <t>20-F FY25</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Sony Music Publishing share of US mechanicals</t>
-        </is>
-      </c>
-      <c r="B37" s="8" t="n">
-        <v>0.26</v>
+          <t>MLC contingency, cumulative to 31 Mar 2026</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>410</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D37" t="inlineStr"/>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Q1-26</t>
+        </is>
+      </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Estimate; SMP ranked #1 publisher in 2025 (range 23-28%)</t>
+          <t>6-K Q1-26 (USD 473M at the time, per NMPA 'nearly $480 million by Spotify's own admission')</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>UMPG direct licence start month (2025)</t>
-        </is>
-      </c>
-      <c r="B38" s="7" t="n">
-        <v>2</v>
+          <t>MLC contingency, cumulative to 30 Jun 2026</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>437</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>month</t>
+          <t>€M</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>2025</t>
+          <t>Q2-26</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Actual</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Announced 26 Jan 2025; reported to 'nullify' the bundle discount going forward</t>
+          <t>6-K Q2-26 as quoted by Music Ally, 7 Sep 2026. A second reading of the same filing gives €473M (which is also the USD value of the Q1-26 figure). Verify against the Q2-26 6-K legal-proceedings note before quoting</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Warner Chappell direct licence start month (2025)</t>
-        </is>
-      </c>
-      <c r="B39" s="7" t="n">
-        <v>3</v>
+          <t>Gross bundle saving 2026E</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>205</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>month</t>
+          <t>€M</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>Reported</t>
+          <t>FY26E</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Announced 6 Feb 2025; 'supersedes the bundling payment structure' (MBW)</t>
+          <t>Placeholder: 4 x average quarterly contingency increment Q2-25 to Q1-26 (€51M). Link to model: bundle saving FY26E</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Sony Music Publishing direct licence start month (2025)</t>
-        </is>
-      </c>
-      <c r="B40" s="7" t="n">
-        <v>10</v>
+          <t>Gross bundle saving 2027E</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="n">
+        <v>205</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>month</t>
+          <t>€M</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>Reported</t>
+          <t>FY27E</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Announced Sep 2025; direct US licence</t>
+          <t>Placeholder: flat on 2026E; Phonorecords IV settlement runs to end-2027. Link to model: bundle saving FY27E</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Share of the bundle discount restored to direct-licensed publishers</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="n">
-        <v>1</v>
+          <t>NMPA estimate of first-year publisher loss</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>230</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr"/>
+          <t>$M</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2024-25</t>
+        </is>
+      </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Assumption per reporting ('nullified'); sensitivity at 50%</t>
+          <t>NMPA via Billboard</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>MLC amended complaint succeeds in 2027 (1 = yes): remaining saving goes to zero</t>
-        </is>
-      </c>
-      <c r="B42" s="9" t="n">
-        <v>0</v>
+          <t>NMPA estimate of cumulative publisher loss to Spotify and Amazon bundling since 2024</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>495</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>flag</t>
+          <t>$M</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>2027</t>
+          <t>Jun-26</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Scenario switch. Interlocutory appeal denied 1 Sep 2026; case continues at district court</t>
+          <t>NMPA annual meeting, Jun 2026 ('nearly $500 million')</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Audiobook licensing cost 2024 ('hundreds of millions of dollars a year' by Oct-24)</t>
-        </is>
-      </c>
-      <c r="B43" s="10" t="n">
-        <v>190</v>
+          <t>Mechanical royalties paid to the MLC, paid tiers, Q4-23</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>97.3</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>€M</t>
+          <t>$M</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>Q4-23</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Axios 15 Oct 2024; Spotify newsroom Mar-25 repeats; 'tens of millions' by Feb-24 (Digital Music News). Sized as a full year</t>
+          <t>Billboard analysis of Spotify's MLC reports</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Audiobook licensing cost growth 2025 (listeners +30-36%, hours +35-37%, DACH launch, Family members)</t>
-        </is>
-      </c>
-      <c r="B44" s="8" t="n">
-        <v>0.58</v>
+          <t>Mechanical royalties paid to the MLC, paid tiers, Q4-25</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>53.3</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>$M</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>Q4-25</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Spotify newsroom Mar-25, Oct-25; estimate</t>
+          <t>Billboard analysis (-45%)</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Audiobook licensing cost growth 2026E (listeners +60%, Nordics, Audiobooks+ Europe)</t>
-        </is>
-      </c>
-      <c r="B45" s="11" t="n">
-        <v>0.43</v>
+          <t>Blended mechanical per-stream rate, paid tiers, Q4-23</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="n">
+        <v>0.00068</v>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>$/stream</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>FY26E</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>LINK TO MODEL</t>
+          <t>Q4-23</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Placeholder: Publishers Weekly 2026. Link to model: audiobook cost growth FY26E</t>
+          <t>Billboard analysis</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Audiobook licensing cost growth 2027E</t>
-        </is>
-      </c>
-      <c r="B46" s="11" t="n">
-        <v>0.3</v>
+          <t>Blended mechanical per-stream rate, paid tiers, Q4-25</t>
+        </is>
+      </c>
+      <c r="B46" s="7" t="n">
+        <v>0.00033</v>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>$/stream</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>FY27E</t>
-        </is>
-      </c>
-      <c r="E46" s="5" t="inlineStr">
-        <is>
-          <t>LINK TO MODEL</t>
+          <t>Q4-25</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Placeholder: assumes deceleration. Link to model: audiobook cost growth FY27E</t>
+          <t>Billboard analysis (-51%)</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Low-case multiplier on audiobook licensing cost</t>
-        </is>
-      </c>
-      <c r="B47" s="12" t="n">
-        <v>0.8</v>
+          <t>EUR/USD, Q4-25 average</t>
+        </is>
+      </c>
+      <c r="B47" s="8" t="n">
+        <v>1.16</v>
       </c>
       <c r="C47" t="inlineStr">
         <is>
           <t>x</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Q4-25</t>
+        </is>
+      </c>
       <c r="E47" t="inlineStr">
         <is>
           <t>Estimate</t>
@@ -1799,115 +1838,103 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Sensitivity band</t>
+          <t>Approximate</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>High-case multiplier on audiobook licensing cost</t>
-        </is>
-      </c>
-      <c r="B48" s="12" t="n">
-        <v>1.25</v>
+          <t>Music share of bundle revenue under CRB allocation</t>
+        </is>
+      </c>
+      <c r="B48" s="6" t="n">
+        <v>0.52</v>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Sensitivity band</t>
+          <t>NMPA / Billboard ('$5.70 of the bundle')</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>US audiobook publisher receipts 2025</t>
-        </is>
-      </c>
-      <c r="B49" s="3" t="n">
-        <v>2430</v>
+          <t>UMPG share of US mechanicals</t>
+        </is>
+      </c>
+      <c r="B49" s="9" t="n">
+        <v>0.22</v>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>$M</t>
-        </is>
-      </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Audio Publishers Association, Jun 2026 (+9%)</t>
+          <t>Estimate from US publishing market shares (range 20-25%)</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>US audiobook publisher receipts 2024</t>
-        </is>
-      </c>
-      <c r="B50" s="3" t="n">
-        <v>2220</v>
+          <t>Warner Chappell share of US mechanicals</t>
+        </is>
+      </c>
+      <c r="B50" s="9" t="n">
+        <v>0.13</v>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>$M</t>
-        </is>
-      </c>
-      <c r="D50" t="inlineStr">
-        <is>
-          <t>FY24</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Audio Publishers Association (+13%)</t>
+          <t>Estimate (range 11-15%)</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Spotify share of US publisher audiobook receipts, low</t>
-        </is>
-      </c>
-      <c r="B51" s="8" t="n">
-        <v>0.1</v>
+          <t>Kobalt share of US mechanicals</t>
+        </is>
+      </c>
+      <c r="B51" s="9" t="n">
+        <v>0.05</v>
       </c>
       <c r="C51" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
+      <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr">
         <is>
           <t>Estimate</t>
@@ -1915,29 +1942,25 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Estimate; Audible 63.4% to 59.8% (eMarketer Mar-26), Spotify #2</t>
+          <t>Estimate; largest independent (range 4-7%)</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Spotify share of US publisher audiobook receipts, high</t>
-        </is>
-      </c>
-      <c r="B52" s="8" t="n">
-        <v>0.14</v>
+          <t>Sony Music Publishing share of US mechanicals</t>
+        </is>
+      </c>
+      <c r="B52" s="9" t="n">
+        <v>0.26</v>
       </c>
       <c r="C52" t="inlineStr">
         <is>
           <t>%</t>
         </is>
       </c>
-      <c r="D52" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
+      <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr">
         <is>
           <t>Estimate</t>
@@ -1945,29 +1968,25 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Estimate; SMP ranked #1 publisher in every quarter of 2025 (range 23-28%)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Non-US markets as a multiple of US cost (UK, AU, CA, IE, NZ, FR, BX, DACH, Nordics)</t>
-        </is>
-      </c>
-      <c r="B53" s="12" t="n">
-        <v>1.4</v>
+          <t>BMG share of US mechanicals</t>
+        </is>
+      </c>
+      <c r="B53" s="9" t="n">
+        <v>0.03</v>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>x</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>FY25</t>
-        </is>
-      </c>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr">
         <is>
           <t>Estimate</t>
@@ -1975,235 +1994,235 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Estimate (range 2-4%)</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>EUR/USD</t>
-        </is>
-      </c>
-      <c r="B54" s="12" t="n">
-        <v>1.13</v>
+          <t>UMPG direct licence start month (2025)</t>
+        </is>
+      </c>
+      <c r="B54" s="10" t="n">
+        <v>2</v>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>x</t>
+          <t>month</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>2025 avg</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Approximate 2025 average</t>
+          <t>Announced 26 Jan 2025; reported to 'nullify' the bundle discount going forward</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Audiobooks+ annual recurring revenue</t>
-        </is>
-      </c>
-      <c r="B55" s="3" t="n">
-        <v>100</v>
+          <t>Warner Chappell direct licence start month (2025)</t>
+        </is>
+      </c>
+      <c r="B55" s="10" t="n">
+        <v>3</v>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>$M</t>
+          <t>month</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Jul-26</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Investor Day 21 May 2026 ('on track for $100M ARR in July'); Q2-26 call: reached</t>
+          <t>Announced 6 Feb 2025; 'supersedes the bundling payment structure' (MBW)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Audiobooks+ paying users</t>
-        </is>
-      </c>
-      <c r="B56" s="13" t="n">
-        <v>1</v>
+          <t>Kobalt direct licence start month (2025)</t>
+        </is>
+      </c>
+      <c r="B56" s="10" t="n">
+        <v>9</v>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>month</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>May-26</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Investor Day via Publishers Weekly ('more than one million')</t>
+          <t>Announced 13 Aug 2025; 'bespoke terms rather than the compulsory licence rates'</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Priced audiobook revenue 2024 (top-ups from Mar-24)</t>
+          <t>Sony Music Publishing direct licence start month (2025)</t>
         </is>
       </c>
       <c r="B57" s="10" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>€M</t>
+          <t>month</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>FY24</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Announced 18 Sep 2025; direct US licence</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Priced audiobook revenue 2025 (US Audiobooks+ from Aug-25; 11 EU markets late-25)</t>
+          <t>BMG direct licence start month (2025)</t>
         </is>
       </c>
       <c r="B58" s="10" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>€M</t>
+          <t>month</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>FY25</t>
+          <t>2025</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Estimate</t>
+          <t>Announced 9 Oct 2025</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Priced audiobook revenue 2026E</t>
-        </is>
-      </c>
-      <c r="B59" s="4" t="n">
-        <v>75</v>
+          <t>Share of the bundle discount restored to direct-licensed publishers</t>
+        </is>
+      </c>
+      <c r="B59" s="9" t="n">
+        <v>0.75</v>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>€M</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>FY26E</t>
-        </is>
-      </c>
-      <c r="E59" s="5" t="inlineStr">
-        <is>
-          <t>LINK TO MODEL</t>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr"/>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Placeholder: ARR $100M mid-year is about €88M run-rate; H1 lower. Link to model: paid audiobook revenue FY26E</t>
+          <t>Estimate. Spotify: liability 'partially offset by direct deals'. MBW on the Warner deal: terms 'continue to recognize a difference between bundled and music-only listeners' but payments 'substantially improved'. Range 50-100%</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Priced audiobook revenue 2027E</t>
-        </is>
-      </c>
-      <c r="B60" s="4" t="n">
-        <v>120</v>
+          <t>MLC amended complaint succeeds in 2027 (1 = yes): the independents' share of the saving goes to zero</t>
+        </is>
+      </c>
+      <c r="B60" s="11" t="n">
+        <v>0</v>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>€M</t>
+          <t>flag</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>FY27E</t>
-        </is>
-      </c>
-      <c r="E60" s="5" t="inlineStr">
-        <is>
-          <t>LINK TO MODEL</t>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Placeholder (+60%). Link to model: paid audiobook revenue FY27E</t>
+          <t>Scenario switch. Interlocutory appeal denied 1 Sep 2026; fact discovery cutoff 13 Mar 2027; no trial date set</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Content cost ratio on paid hours (same publisher payments apply)</t>
-        </is>
-      </c>
-      <c r="B61" s="8" t="n">
-        <v>0.55</v>
+          <t>Audiobook licensing cost 2024 ('hundreds of millions of dollars a year' by Oct-24)</t>
+        </is>
+      </c>
+      <c r="B61" s="12" t="n">
+        <v>190</v>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr"/>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
       <c r="E61" t="inlineStr">
         <is>
           <t>Estimate</t>
@@ -2211,78 +2230,78 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Assumption</t>
+          <t>Axios 15 Oct 2024; Spotify newsroom Mar-25 repeats; 'tens of millions' by Feb-24 (Digital Music News). Sized as a full year</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>Premium subscribers</t>
-        </is>
-      </c>
-      <c r="B62" s="13" t="n">
-        <v>300</v>
+          <t>Audiobook licensing cost growth 2025 (listeners +30-36%, hours +35-37%, DACH launch, Family members)</t>
+        </is>
+      </c>
+      <c r="B62" s="9" t="n">
+        <v>0.58</v>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Q2-26</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Spotify Q2-26 deck</t>
+          <t>Spotify newsroom Mar-25, Oct-25; estimate</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>Subscribers in markets with audiobooks in Premium</t>
-        </is>
-      </c>
-      <c r="B63" s="14" t="n">
-        <v>140</v>
+          <t>Audiobook licensing cost growth 2026E (listeners +60%, Nordics, Audiobooks+ Europe)</t>
+        </is>
+      </c>
+      <c r="B63" s="13" t="n">
+        <v>0.43</v>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Q2-26</t>
-        </is>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>Estimate</t>
+          <t>FY26E</t>
+        </is>
+      </c>
+      <c r="E63" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Estimate: North America 75M + eligible Europe ~60M + AU/NZ ~6M</t>
+          <t>Placeholder: Publishers Weekly 2026. Link to model: audiobook cost growth FY26E</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>Share of Premium subscribers listening to audiobooks</t>
-        </is>
-      </c>
-      <c r="B64" s="6" t="n">
-        <v>0.25</v>
+          <t>Audiobook licensing cost growth 2027E</t>
+        </is>
+      </c>
+      <c r="B64" s="13" t="n">
+        <v>0.3</v>
       </c>
       <c r="C64" t="inlineStr">
         <is>
@@ -2291,187 +2310,179 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>2025</t>
-        </is>
-      </c>
-      <c r="E64" t="inlineStr">
-        <is>
-          <t>Reported</t>
+          <t>FY27E</t>
+        </is>
+      </c>
+      <c r="E64" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>The Bookseller 2025; TechCrunch 17 Jul 2025</t>
+          <t>Placeholder: assumes deceleration. Link to model: audiobook cost growth FY27E</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Share of eligible Premium users who have ever pressed play</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="n">
-        <v>0.5</v>
+          <t>Low-case multiplier on audiobook licensing cost</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="n">
+        <v>0.8</v>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>Oct-25</t>
-        </is>
-      </c>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Spotify newsroom 15 Oct 2025</t>
+          <t>Sensitivity band</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>US individual subscribers who took the $1 Basic plan to drop audiobooks</t>
-        </is>
-      </c>
-      <c r="B66" s="6" t="n">
-        <v>0.155</v>
+          <t>High-case multiplier on audiobook licensing cost</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="n">
+        <v>1.25</v>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>2024</t>
-        </is>
-      </c>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr">
         <is>
-          <t>Reported</t>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Morgan Stanley survey via Billboard (14-17%)</t>
+          <t>Sensitivity band</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Music Pro attach assumption, bull case</t>
-        </is>
-      </c>
-      <c r="B67" s="11" t="n">
-        <v>0.03</v>
+          <t>US audiobook publisher receipts 2025</t>
+        </is>
+      </c>
+      <c r="B67" s="3" t="n">
+        <v>2430</v>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>%</t>
+          <t>$M</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>2027</t>
-        </is>
-      </c>
-      <c r="E67" s="5" t="inlineStr">
-        <is>
-          <t>LINK TO MODEL</t>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Placeholder. Link to model: bull-case Music Pro attach</t>
+          <t>Audio Publishers Association, Jun 2026 (+9%)</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>Consensus gross-margin expansion 2026E</t>
-        </is>
-      </c>
-      <c r="B68" s="15" t="n">
-        <v>115</v>
+          <t>US audiobook publisher receipts 2024</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="n">
+        <v>2220</v>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>bp</t>
+          <t>$M</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>FY26E</t>
-        </is>
-      </c>
-      <c r="E68" s="5" t="inlineStr">
-        <is>
-          <t>LINK TO MODEL</t>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Reported</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Placeholder: 33.2% vs 32.0%. Link to model: consensus gross margin FY26E</t>
+          <t>Audio Publishers Association (+13%)</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Consensus gross-margin expansion 2027E</t>
-        </is>
-      </c>
-      <c r="B69" s="15" t="n">
-        <v>130</v>
+          <t>Spotify share of US publisher audiobook receipts, low</t>
+        </is>
+      </c>
+      <c r="B69" s="9" t="n">
+        <v>0.1</v>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>bp</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>FY27E</t>
-        </is>
-      </c>
-      <c r="E69" s="5" t="inlineStr">
-        <is>
-          <t>LINK TO MODEL</t>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>Estimate</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Placeholder: ~34.5% vs 33.2%. Link to model: consensus gross margin FY27E</t>
+          <t>Estimate; Audible 63.4% to 59.8% (eMarketer Mar-26), Spotify #2</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Memo: Jun-24 US price increase, annualized revenue (not in N)</t>
-        </is>
-      </c>
-      <c r="B70" s="10" t="n">
-        <v>500</v>
+          <t>Spotify share of US publisher audiobook receipts, high</t>
+        </is>
+      </c>
+      <c r="B70" s="9" t="n">
+        <v>0.14</v>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>€M</t>
+          <t>%</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>run-rate</t>
+          <t>FY25</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2481,124 +2492,660 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Estimate: ~7% blended on ~€8B US Premium revenue</t>
+          <t>Estimate</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Non-US markets as a multiple of US cost (UK, AU, CA, IE, NZ, FR, BX, DACH, Nordics)</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Estimate</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="16" t="inlineStr">
-        <is>
-          <t>Sources</t>
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="B72" s="8" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>x</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>2025 avg</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Approximate 2025 average</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>Spotify Form 6-K, Q1-25 (bundle: ~€205M additional royalties for 1 Mar 2024–31 Mar 2025 if the MLC prevailed): sec.gov/Archives/edgar/data/1639920/000163992025000006/spot-20250331x6xk.htm</t>
+          <t>Audiobooks+ annual recurring revenue</t>
+        </is>
+      </c>
+      <c r="B73" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>$M</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Jul-26</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Investor Day 21 May 2026 ('on track for $100M ARR in July'); Q2-26 call: reached</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Spotify Form 20-F FY2024 and FY2025 (Premium cost of revenue drivers, royalty component increases, Premium GM): sec.gov/Archives/edgar/data/1639920/000163992025000003/ck0001639920-20241231.htm ; .../000162828026006874/ck0001639920-20251231.htm</t>
+          <t>Audiobooks+ paying users</t>
+        </is>
+      </c>
+      <c r="B74" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>May-26</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Investor Day via Publishers Weekly ('more than one million')</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Spotify Form 6-K Q2-26 (H1-26 Premium cost of revenue +€500M, content +€474M, ratio 67%→65%): sec.gov/Archives/edgar/data/0001639920/000162828026052543/spot-20260630x6xk.htm</t>
+          <t>Priced audiobook revenue 2024 (top-ups from Mar-24)</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>FY24</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Estimate</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Spotify Form 6-K Q3-25 (9M-25 royalty component +€588M): sec.gov/Archives/edgar/data/1639920/000162828025048927/spot-20250930x6xk.htm</t>
+          <t>Priced audiobook revenue 2025 (US Audiobooks+ from Aug-25; 11 EU markets late-25)</t>
+        </is>
+      </c>
+      <c r="B76" s="12" t="n">
+        <v>30</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>FY25</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Estimate</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Billboard, 'How much have Spotify bundles decreased the mechanical per-stream rate' (Q4-23 $97.3M → Q4-25 $53.3M; per-stream −51%)</t>
+          <t>Priced audiobook revenue 2026E</t>
+        </is>
+      </c>
+      <c r="B77" s="4" t="n">
+        <v>75</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>FY26E</t>
+        </is>
+      </c>
+      <c r="E77" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Placeholder: ARR $100M mid-year is about €88M run-rate; H1 lower. Link to model: paid audiobook revenue FY26E</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>NMPA statements: $150M (May 2024), $230M first-year loss, ~$500M cumulative with Amazon (2025–26); Billboard 'bundling controversy one year later'</t>
+          <t>Priced audiobook revenue 2027E</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>FY27E</t>
+        </is>
+      </c>
+      <c r="E78" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Placeholder (+60%). Link to model: paid audiobook revenue FY27E</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>Direct deals: UMPG (26 Jan 2025, DMN/Billboard: bundle discount 'nullified going forward'); Warner Chappell (6 Feb 2025, MBW: 'supersedes the bundling payment structure'); Sony Music Publishing (Sep 2025, MBW)</t>
+          <t>Content cost ratio on paid hours (same publisher payments apply)</t>
+        </is>
+      </c>
+      <c r="B79" s="9" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr"/>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Assumption</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>MLC v. Spotify: dismissal Jan 2025 (Variety); amended complaint late 2025; interlocutory appeal denied 1 Sep 2026 (MBW, Soundstock)</t>
+          <t>Premium subscribers</t>
+        </is>
+      </c>
+      <c r="B80" s="14" t="n">
+        <v>300</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>Q2-26</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Spotify Q2-26 deck</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Audiobook cost phrases: Digital Music News 5 Feb 2024 ('tens of millions'); Axios 15 Oct 2024 ('hundreds of millions annually'); Spotify newsroom 13 Mar 2025</t>
+          <t>Subscribers in markets with audiobooks in Premium</t>
+        </is>
+      </c>
+      <c r="B81" s="15" t="n">
+        <v>140</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>Q2-26</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Estimate: North America 75M + eligible Europe ~60M + AU/NZ ~6M</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Spotify newsroom 15 Oct 2025 (two-year stats: listeners +36%, hours +37%, &gt;50% tried); Mar 2025 (listeners +30%, hours +35%, 400k titles); Publishers Weekly 2026 (listeners +60%, Audiobooks+ $100M ARR, &gt;1M payers)</t>
+          <t>Share of Premium subscribers listening to audiobooks</t>
+        </is>
+      </c>
+      <c r="B82" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>The Bookseller 2025; TechCrunch 17 Jul 2025</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>The Bookseller 2025 / TechCrunch 17 Jul 2025 ('more than 25% of Premium subscribers listening')</t>
+          <t>Share of eligible Premium users who have ever pressed play</t>
+        </is>
+      </c>
+      <c r="B83" s="6" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>Oct-25</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Spotify newsroom 15 Oct 2025</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Audio Publishers Association sales surveys: 2022 $1.8B, 2023 $2.0B, 2024 $2.22B, 2025 $2.43B; eMarketer Mar 2026 (Audible 63.4%→59.8%)</t>
+          <t>US individual subscribers who took the $1 Basic plan to drop audiobooks</t>
+        </is>
+      </c>
+      <c r="B84" s="6" t="n">
+        <v>0.155</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>Reported</t>
+        </is>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>Morgan Stanley survey via Billboard (14-17%)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Publisher confirmations: Bloomsbury AR 2025 (audio +57% 'in part Spotify'); News Corp/HarperCollins (audio +18% FY, +28% Q4, citing Spotify)</t>
+          <t>Music Pro attach assumption, bull case</t>
+        </is>
+      </c>
+      <c r="B85" s="13" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>%</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>2027</t>
+        </is>
+      </c>
+      <c r="E85" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Placeholder. Link to model: bull-case Music Pro attach</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Audible Standard plan $8.99 (Audible newsroom, 3 Mar 2026); Amazon Music Unlimited + Audible (Nov 2024)</t>
+          <t>Consensus gross-margin expansion 2026E</t>
+        </is>
+      </c>
+      <c r="B86" s="16" t="n">
+        <v>115</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>bp</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>FY26E</t>
+        </is>
+      </c>
+      <c r="E86" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
+        </is>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>Placeholder: 33.2% vs 32.0%. Link to model: consensus gross margin FY26E</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Basic plan opt-out 14–17% (Morgan Stanley survey via Billboard, 2024)</t>
+          <t>Consensus gross-margin expansion 2027E</t>
+        </is>
+      </c>
+      <c r="B87" s="16" t="n">
+        <v>130</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>bp</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>FY27E</t>
+        </is>
+      </c>
+      <c r="E87" s="5" t="inlineStr">
+        <is>
+          <t>LINK TO MODEL</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Placeholder: ~34.5% vs 33.2%. Link to model: consensus gross margin FY27E</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
+        <is>
+          <t>Memo: Jun-24 US price increase, annualized revenue (not in N)</t>
+        </is>
+      </c>
+      <c r="B88" s="12" t="n">
+        <v>500</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>€M</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>run-rate</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Estimate</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Estimate: ~7% blended on ~€8B US Premium revenue</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="17" t="inlineStr">
+        <is>
+          <t>Sources</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>MLC contingency series (legal proceedings note in each filing): 6-K Q2-24 sec.gov/Archives/edgar/data/1639920/000163992024000009/spot-20240630x6xk.htm; 6-K Q3-24 .../000163992024000013/spot-20240930x6xk.htm; 20-F FY24 .../000163992025000003/ck0001639920-20241231.htm; 6-K Q1-25 .../000163992025000006/spot-20250331x6xk.htm; 6-K Q2-25 .../000163992025000012/spot-20250630x6xk.htm; 6-K Q3-25 .../000162828025048927/spot-20250930x6xk.htm; 20-F FY25 .../000162828026006874/ck0001639920-20251231.htm; 6-K Q1-26 .../000162828026027951/spot-20260331x6xk.htm; 6-K Q2-26 .../000162828026052543/spot-20260630x6xk.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Billboard, 'How Much Have Spotify Bundles Decreased the Mechanical Per-Stream Rate? (Analysis)': Q4-23 $97.3M at $0.00068 per stream; Q4-25 $53.3M at $0.00033; streams +19.3bn</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Direct deals: UMPG 26 Jan 2025 (MBW); Warner Chappell 6 Feb 2025 (MBW: 'supersedes the bundling payment structure'; terms 'continue to recognize a difference between bundled and music-only listeners'); Kobalt 13 Aug 2025 (CMU, MBW); Sony Music Publishing 18 Sep 2025 (MBW, Variety); BMG 9 Oct 2025 (CMU)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>MLC v. Spotify USA Inc., S.D.N.Y. 1:24-cv-03809: dismissed with prejudice 29 Jan 2025; reconsideration granted Sep 2025; amended complaint 1 Oct 2025 (valuation of the bundle components and the Audiobook Access tier); jury demand 8 Oct 2025; interlocutory appeal denied 1 Sep 2026; fact discovery cutoff 13 Mar 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Spotify Form 20-F FY2024 and FY2025 (Premium cost of revenue drivers, royalty component increases, Premium GM): sec.gov/Archives/edgar/data/1639920/000163992025000003/ck0001639920-20241231.htm ; .../000162828026006874/ck0001639920-20251231.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Spotify Form 6-K Q2-26 (H1-26 Premium cost of revenue +€500M, content +€474M, ratio 67%→65%): sec.gov/Archives/edgar/data/0001639920/000162828026052543/spot-20260630x6xk.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Spotify Form 6-K Q3-25 (9M-25 royalty component +€588M): sec.gov/Archives/edgar/data/1639920/000162828025048927/spot-20250930x6xk.htm</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>NMPA statements: $150M (May 2024), $230M first-year loss, nearly $500M cumulative with Amazon (annual meeting, Jun 2026; 'nearly $480 million by Spotify's own admission')</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Audiobook cost phrases: Digital Music News 5 Feb 2024 ('tens of millions'); Axios 15 Oct 2024 ('hundreds of millions annually'); Spotify newsroom 13 Mar 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Spotify newsroom 15 Oct 2025 (two-year stats: listeners +36%, hours +37%, &gt;50% tried); Mar 2025 (listeners +30%, hours +35%, 400k titles); Publishers Weekly 2026 (listeners +60%, Audiobooks+ $100M ARR, &gt;1M payers)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>The Bookseller 2025 / TechCrunch 17 Jul 2025 ('more than 25% of Premium subscribers listening')</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Audio Publishers Association sales surveys: 2022 $1.8B, 2023 $2.0B, 2024 $2.22B, 2025 $2.43B; eMarketer Mar 2026 (Audible 63.4%→59.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Publisher confirmations: Bloomsbury AR 2025 (audio +57% 'in part Spotify'); News Corp/HarperCollins (audio +18% FY, +28% Q4, citing Spotify)</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Audible Standard plan $8.99 (Audible newsroom, 3 Mar 2026); Amazon Music Unlimited + Audible (Nov 2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Basic plan opt-out 14–17% (Morgan Stanley survey via Billboard, 2024)</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
         <is>
           <t>Audiobooks+ launch and pricing: 9to5Mac 5 Aug 2025; Publishers Weekly (11 EU markets); Spotify newsroom Mar 2024 (Access tier, top-ups)</t>
         </is>
@@ -2615,7 +3162,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F88"/>
+  <dimension ref="A1:F117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="88" customWidth="1" min="1" max="1"/>
@@ -2645,356 +3192,359 @@
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="17" t="n"/>
-      <c r="C4" s="18" t="inlineStr">
+      <c r="B4" s="18" t="n"/>
+      <c r="C4" s="19" t="inlineStr">
         <is>
           <t>2024A</t>
         </is>
       </c>
-      <c r="D4" s="18" t="inlineStr">
+      <c r="D4" s="19" t="inlineStr">
         <is>
           <t>2025A</t>
         </is>
       </c>
-      <c r="E4" s="18" t="inlineStr">
+      <c r="E4" s="19" t="inlineStr">
         <is>
           <t>2026E</t>
         </is>
       </c>
-      <c r="F4" s="18" t="inlineStr">
+      <c r="F4" s="19" t="inlineStr">
         <is>
           <t>2027E</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>1. Bundle mechanical-royalty saving (B)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Run-rate bundle saving, €M per year (13-month disclosure x 12/13)</t>
-        </is>
-      </c>
-      <c r="B6" s="19">
-        <f>Audiobooks_Inputs!$B$29/Audiobooks_Inputs!$B$30*12</f>
-        <v/>
+      <c r="A6" s="17" t="inlineStr">
+        <is>
+          <t>a. MLC contingency disclosed in Spotify filings: additional royalties due if Premium were not a bundle, cumulative from 1 Mar 2024 (€M)</t>
+        </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Months bundle active in year</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="n">
-        <v>10</v>
-      </c>
-      <c r="D7" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="E7" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <v>12</v>
+      <c r="A7" s="17" t="inlineStr">
+        <is>
+          <t>Filing (period end)</t>
+        </is>
+      </c>
+      <c r="C7" s="20" t="inlineStr">
+        <is>
+          <t>Cumulative</t>
+        </is>
+      </c>
+      <c r="D7" s="20" t="inlineStr">
+        <is>
+          <t>Increment</t>
+        </is>
+      </c>
+      <c r="E7" s="20" t="inlineStr">
+        <is>
+          <t>Months</t>
+        </is>
+      </c>
+      <c r="F7" s="20" t="inlineStr">
+        <is>
+          <t>€M per month</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Gross saving = run-rate x months / 12</t>
-        </is>
-      </c>
-      <c r="C8" s="20">
-        <f>$B$6*C7/12</f>
-        <v/>
-      </c>
-      <c r="D8" s="20">
-        <f>$B$6*D7/12</f>
-        <v/>
-      </c>
-      <c r="E8" s="20">
-        <f>$B$6*E7/12</f>
-        <v/>
-      </c>
-      <c r="F8" s="20">
-        <f>$B$6*F7/12</f>
+          <t>6-K Q2-24 (30 Jun 2024)</t>
+        </is>
+      </c>
+      <c r="C8" s="21">
+        <f>Audiobooks_Inputs!$B$29</f>
+        <v/>
+      </c>
+      <c r="D8" s="22">
+        <f>C8</f>
+        <v/>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F8" s="23">
+        <f>D8/E8</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>UMPG months on direct licence</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="21">
-        <f>13-Audiobooks_Inputs!$B$38</f>
-        <v/>
-      </c>
-      <c r="E9" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="F9" s="7" t="n">
-        <v>12</v>
+          <t>6-K Q3-24 (30 Sep 2024)</t>
+        </is>
+      </c>
+      <c r="C9" s="21">
+        <f>Audiobooks_Inputs!$B$31</f>
+        <v/>
+      </c>
+      <c r="D9" s="22">
+        <f>C9-C8</f>
+        <v/>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F9" s="23">
+        <f>D9/E9</f>
+        <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Warner Chappell months on direct licence</t>
-        </is>
-      </c>
-      <c r="C10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="21">
-        <f>13-Audiobooks_Inputs!$B$39</f>
-        <v/>
-      </c>
-      <c r="E10" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="F10" s="7" t="n">
-        <v>12</v>
+          <t>20-F FY24 (31 Dec 2024)</t>
+        </is>
+      </c>
+      <c r="C10" s="21">
+        <f>Audiobooks_Inputs!$B$32</f>
+        <v/>
+      </c>
+      <c r="D10" s="22">
+        <f>C10-C9</f>
+        <v/>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F10" s="23">
+        <f>D10/E10</f>
+        <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Sony Music Publishing months on direct licence</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="21">
-        <f>13-Audiobooks_Inputs!$B$40</f>
-        <v/>
-      </c>
-      <c r="E11" s="7" t="n">
-        <v>12</v>
-      </c>
-      <c r="F11" s="7" t="n">
-        <v>12</v>
+          <t>6-K Q1-25 (31 Mar 2025)</t>
+        </is>
+      </c>
+      <c r="C11" s="21">
+        <f>Audiobooks_Inputs!$B$33</f>
+        <v/>
+      </c>
+      <c r="D11" s="22">
+        <f>C11-C10</f>
+        <v/>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F11" s="23">
+        <f>D11/E11</f>
+        <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Hand-back to direct-licensed publishers = run-rate x sum(share x months / 12) x restoration</t>
-        </is>
-      </c>
-      <c r="C12" s="19">
-        <f>$B$6*(Audiobooks_Inputs!$B$35*C9+Audiobooks_Inputs!$B$36*C10+Audiobooks_Inputs!$B$37*C11)/12*Audiobooks_Inputs!$B$41</f>
-        <v/>
-      </c>
-      <c r="D12" s="19">
-        <f>$B$6*(Audiobooks_Inputs!$B$35*D9+Audiobooks_Inputs!$B$36*D10+Audiobooks_Inputs!$B$37*D11)/12*Audiobooks_Inputs!$B$41</f>
-        <v/>
-      </c>
-      <c r="E12" s="19">
-        <f>$B$6*(Audiobooks_Inputs!$B$35*E9+Audiobooks_Inputs!$B$36*E10+Audiobooks_Inputs!$B$37*E11)/12*Audiobooks_Inputs!$B$41</f>
-        <v/>
-      </c>
-      <c r="F12" s="19">
-        <f>$B$6*(Audiobooks_Inputs!$B$35*F9+Audiobooks_Inputs!$B$36*F10+Audiobooks_Inputs!$B$37*F11)/12*Audiobooks_Inputs!$B$41</f>
+          <t>6-K Q2-25 (30 Jun 2025)</t>
+        </is>
+      </c>
+      <c r="C12" s="21">
+        <f>Audiobooks_Inputs!$B$34</f>
+        <v/>
+      </c>
+      <c r="D12" s="22">
+        <f>C12-C11</f>
+        <v/>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F12" s="23">
+        <f>D12/E12</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
-        <is>
-          <t>B  Net bundle saving (2027: zero if MLC switch = 1)</t>
-        </is>
-      </c>
-      <c r="C13" s="20">
-        <f>C8-C12</f>
-        <v/>
-      </c>
-      <c r="D13" s="20">
-        <f>D8-D12</f>
-        <v/>
-      </c>
-      <c r="E13" s="20">
-        <f>E8-E12</f>
-        <v/>
-      </c>
-      <c r="F13" s="19">
-        <f>IF(Audiobooks_Inputs!$B$42=1,0,F8-F12)</f>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>6-K Q3-25 (30 Sep 2025)</t>
+        </is>
+      </c>
+      <c r="C13" s="21">
+        <f>Audiobooks_Inputs!$B$35</f>
+        <v/>
+      </c>
+      <c r="D13" s="22">
+        <f>C13-C12</f>
+        <v/>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F13" s="23">
+        <f>D13/E13</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>20-F FY25 (31 Dec 2025)</t>
+        </is>
+      </c>
+      <c r="C14" s="21">
+        <f>Audiobooks_Inputs!$B$36</f>
+        <v/>
+      </c>
+      <c r="D14" s="22">
+        <f>C14-C13</f>
+        <v/>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F14" s="23">
+        <f>D14/E14</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
-        <is>
-          <t>2. Audiobook licensing cost on included hours (C)</t>
-        </is>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>6-K Q1-26 (31 Mar 2026)</t>
+        </is>
+      </c>
+      <c r="C15" s="21">
+        <f>Audiobooks_Inputs!$B$37</f>
+        <v/>
+      </c>
+      <c r="D15" s="22">
+        <f>C15-C14</f>
+        <v/>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F15" s="23">
+        <f>D15/E15</f>
+        <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Growth y/y</t>
-        </is>
+          <t>6-K Q2-26 (30 Jun 2026): verify, see inputs note</t>
+        </is>
+      </c>
+      <c r="C16" s="21">
+        <f>Audiobooks_Inputs!$B$38</f>
+        <v/>
       </c>
       <c r="D16" s="22">
-        <f>Audiobooks_Inputs!$B$44</f>
-        <v/>
-      </c>
-      <c r="E16" s="22">
-        <f>Audiobooks_Inputs!$B$45</f>
-        <v/>
-      </c>
-      <c r="F16" s="22">
-        <f>Audiobooks_Inputs!$B$46</f>
+        <f>C16-C15</f>
+        <v/>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" s="23">
+        <f>D16/E16</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
-        <is>
-          <t>C  Base case</t>
-        </is>
-      </c>
-      <c r="C17" s="19">
-        <f>Audiobooks_Inputs!$B$43</f>
-        <v/>
-      </c>
-      <c r="D17" s="20">
-        <f>C17*(1+D16)</f>
-        <v/>
-      </c>
-      <c r="E17" s="20">
-        <f>D17*(1+E16)</f>
-        <v/>
-      </c>
-      <c r="F17" s="20">
-        <f>E17*(1+F16)</f>
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   of which April to June 2024 (so March 2024 alone was about €11M)</t>
+        </is>
+      </c>
+      <c r="C17" s="21">
+        <f>Audiobooks_Inputs!$B$30</f>
+        <v/>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F17" s="23">
+        <f>C17/E17</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>C  Low case</t>
-        </is>
-      </c>
-      <c r="C18" s="19">
-        <f>C17*Audiobooks_Inputs!$B$47</f>
-        <v/>
-      </c>
-      <c r="D18" s="19">
-        <f>D17*Audiobooks_Inputs!$B$47</f>
-        <v/>
-      </c>
-      <c r="E18" s="19">
-        <f>E17*Audiobooks_Inputs!$B$47</f>
-        <v/>
-      </c>
-      <c r="F18" s="19">
-        <f>F17*Audiobooks_Inputs!$B$47</f>
+          <t>Average quarterly increment, Q2-25 to Q1-26</t>
+        </is>
+      </c>
+      <c r="B18" s="23">
+        <f>AVERAGE(D12:D15)</f>
         <v/>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>C  High case</t>
-        </is>
-      </c>
-      <c r="C19" s="19">
-        <f>C17*Audiobooks_Inputs!$B$48</f>
-        <v/>
-      </c>
-      <c r="D19" s="19">
-        <f>D17*Audiobooks_Inputs!$B$48</f>
-        <v/>
-      </c>
-      <c r="E19" s="19">
-        <f>E17*Audiobooks_Inputs!$B$48</f>
-        <v/>
-      </c>
-      <c r="F19" s="19">
-        <f>F17*Audiobooks_Inputs!$B$48</f>
+          <t>Annualised</t>
+        </is>
+      </c>
+      <c r="B19" s="22">
+        <f>B18*4</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Reading: the increment ran at €50-56M a quarter from Q4-24 to Q1-26 with no step down after the direct deals, so the figure is gross: Spotify still reports every paid-tier stream through the MLC at the bundle rate and pays the direct-licensed publishers a top-up outside it. The Q2-26 increment of €27M is either an FX translation effect or the first filing to net out direct-deal publishers; the 6-K wording decides which.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
-        <is>
-          <t>3. Priced channel (Audiobooks+, top-ups, a la carte)</t>
-        </is>
-      </c>
+      <c r="A21" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>Revenue</t>
-        </is>
-      </c>
-      <c r="C22" s="19">
-        <f>Audiobooks_Inputs!$B$57</f>
-        <v/>
-      </c>
-      <c r="D22" s="19">
-        <f>Audiobooks_Inputs!$B$58</f>
-        <v/>
-      </c>
-      <c r="E22" s="19">
-        <f>Audiobooks_Inputs!$B$59</f>
-        <v/>
-      </c>
-      <c r="F22" s="19">
-        <f>Audiobooks_Inputs!$B$60</f>
-        <v/>
+      <c r="A22" s="17" t="inlineStr">
+        <is>
+          <t>b. Gross bundle saving by year</t>
+        </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>Content cost ratio on paid hours</t>
-        </is>
-      </c>
-      <c r="B23" s="22">
-        <f>Audiobooks_Inputs!$B$61</f>
+      <c r="A23" s="17" t="inlineStr">
+        <is>
+          <t>Gross saving (2024-25 from filings; 2026E-27E placeholders on the inputs tab)</t>
+        </is>
+      </c>
+      <c r="C23" s="21">
+        <f>Audiobooks_Inputs!$B$32</f>
+        <v/>
+      </c>
+      <c r="D23" s="21">
+        <f>Audiobooks_Inputs!$B$36-Audiobooks_Inputs!$B$32</f>
+        <v/>
+      </c>
+      <c r="E23" s="21">
+        <f>Audiobooks_Inputs!$B$39</f>
+        <v/>
+      </c>
+      <c r="F23" s="21">
+        <f>Audiobooks_Inputs!$B$40</f>
         <v/>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
-        <is>
-          <t>A  Gross profit on paid hours = revenue x (1 - ratio)</t>
-        </is>
-      </c>
-      <c r="C24" s="20">
-        <f>C22*(1-$B$23)</f>
-        <v/>
-      </c>
-      <c r="D24" s="20">
-        <f>D22*(1-$B$23)</f>
-        <v/>
-      </c>
-      <c r="E24" s="20">
-        <f>E22*(1-$B$23)</f>
-        <v/>
-      </c>
-      <c r="F24" s="20">
-        <f>F22*(1-$B$23)</f>
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>NMPA: first-year loss $230M; cumulative to Jun-26 (with Amazon) nearly $500M</t>
+        </is>
+      </c>
+      <c r="B24" s="21">
+        <f>Audiobooks_Inputs!$B$41</f>
+        <v/>
+      </c>
+      <c r="C24" s="21">
+        <f>Audiobooks_Inputs!$B$42</f>
         <v/>
       </c>
     </row>
@@ -3002,645 +3552,768 @@
       <c r="A25" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
-        <is>
-          <t>4. Net contribution to gross profit: N = B + A - C</t>
+      <c r="A26" s="17" t="inlineStr">
+        <is>
+          <t>c. Cross-check: Billboard analysis of Spotify's MLC reports, paid tiers</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>B  Net bundle saving</t>
-        </is>
-      </c>
-      <c r="C27" s="20">
-        <f>C13</f>
-        <v/>
-      </c>
-      <c r="D27" s="20">
-        <f>D13</f>
-        <v/>
-      </c>
-      <c r="E27" s="20">
-        <f>E13</f>
-        <v/>
-      </c>
-      <c r="F27" s="20">
-        <f>F13</f>
+          <t>Mechanical royalties paid to the MLC, $M: Q4-23 (col B), Q4-25 (col C)</t>
+        </is>
+      </c>
+      <c r="B27" s="24">
+        <f>Audiobooks_Inputs!$B$43</f>
+        <v/>
+      </c>
+      <c r="C27" s="24">
+        <f>Audiobooks_Inputs!$B$44</f>
         <v/>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>A  Gross profit on paid hours</t>
-        </is>
-      </c>
-      <c r="C28" s="20">
-        <f>C24</f>
-        <v/>
-      </c>
-      <c r="D28" s="20">
-        <f>D24</f>
-        <v/>
-      </c>
-      <c r="E28" s="20">
-        <f>E24</f>
-        <v/>
-      </c>
-      <c r="F28" s="20">
-        <f>F24</f>
+          <t>Blended per-stream rate, $: Q4-23 (col B), Q4-25 (col C)</t>
+        </is>
+      </c>
+      <c r="B28" s="25">
+        <f>Audiobooks_Inputs!$B$45</f>
+        <v/>
+      </c>
+      <c r="C28" s="25">
+        <f>Audiobooks_Inputs!$B$46</f>
         <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>C  Licensing cost on included hours</t>
-        </is>
-      </c>
-      <c r="C29" s="20">
-        <f>C17</f>
-        <v/>
-      </c>
-      <c r="D29" s="20">
-        <f>D17</f>
-        <v/>
-      </c>
-      <c r="E29" s="20">
-        <f>E17</f>
-        <v/>
-      </c>
-      <c r="F29" s="20">
-        <f>F17</f>
+          <t>Implied paid-tier streams, bn: Q4-23 (col B), Q4-25 (col C)</t>
+        </is>
+      </c>
+      <c r="B29" s="23">
+        <f>B27/B28/1000</f>
+        <v/>
+      </c>
+      <c r="C29" s="23">
+        <f>C27/C28/1000</f>
         <v/>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="16" t="inlineStr">
-        <is>
-          <t>N  Net contribution</t>
-        </is>
-      </c>
-      <c r="C30" s="20">
-        <f>C27+C28-C29</f>
-        <v/>
-      </c>
-      <c r="D30" s="20">
-        <f>D27+D28-D29</f>
-        <v/>
-      </c>
-      <c r="E30" s="20">
-        <f>E27+E28-E29</f>
-        <v/>
-      </c>
-      <c r="F30" s="20">
-        <f>F27+F28-F29</f>
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Counterfactual Q4-25 payment at the Q4-23 rate, $M</t>
+        </is>
+      </c>
+      <c r="B30" s="23">
+        <f>C29*B28*1000</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Group revenue</t>
-        </is>
-      </c>
-      <c r="C31" s="19">
-        <f>Audiobooks_Inputs!$B$12</f>
-        <v/>
-      </c>
-      <c r="D31" s="19">
-        <f>Audiobooks_Inputs!$B$13</f>
-        <v/>
-      </c>
-      <c r="E31" s="19">
-        <f>Audiobooks_Inputs!$B$14</f>
-        <v/>
-      </c>
-      <c r="F31" s="19">
-        <f>Audiobooks_Inputs!$B$15</f>
+          <t>Implied quarterly bundle discount, $M</t>
+        </is>
+      </c>
+      <c r="B31" s="23">
+        <f>B30-C27</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>N, bp of group revenue</t>
-        </is>
-      </c>
-      <c r="C32" s="23">
-        <f>C30/C31*10000</f>
-        <v/>
-      </c>
-      <c r="D32" s="23">
-        <f>D30/D31*10000</f>
-        <v/>
-      </c>
-      <c r="E32" s="23">
-        <f>E30/E31*10000</f>
-        <v/>
-      </c>
-      <c r="F32" s="23">
-        <f>F30/F31*10000</f>
+          <t>EUR/USD, Q4-25</t>
+        </is>
+      </c>
+      <c r="B32" s="26">
+        <f>Audiobooks_Inputs!$B$47</f>
         <v/>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="16" t="inlineStr">
-        <is>
-          <t>Change in N y/y, €M (gross-margin headwind)</t>
-        </is>
-      </c>
-      <c r="D33" s="20">
-        <f>D30-C30</f>
-        <v/>
-      </c>
-      <c r="E33" s="20">
-        <f>E30-D30</f>
-        <v/>
-      </c>
-      <c r="F33" s="20">
-        <f>F30-E30</f>
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Implied quarterly discount, €M (col B) vs 6-K Q4-25 increment (col C)</t>
+        </is>
+      </c>
+      <c r="B33" s="23">
+        <f>B31/B32</f>
+        <v/>
+      </c>
+      <c r="C33" s="23">
+        <f>D14</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="16" t="inlineStr">
-        <is>
-          <t>Change in N y/y, bp of group revenue</t>
-        </is>
-      </c>
-      <c r="D34" s="23">
-        <f>D33/D31*10000</f>
-        <v/>
-      </c>
-      <c r="E34" s="23">
-        <f>E33/E31*10000</f>
-        <v/>
-      </c>
-      <c r="F34" s="23">
-        <f>F33/F31*10000</f>
-        <v/>
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Reading: streams in the MLC reports grew 19bn between the two quarters, so direct-licensed publishers have not left the blanket licence. Two independent sources put the gross discount at about €50M a quarter.</t>
+        </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   of which music publishers reclaim the bundle saving (change in B)</t>
-        </is>
-      </c>
-      <c r="D35" s="20">
-        <f>D27-C27</f>
-        <v/>
-      </c>
-      <c r="E35" s="20">
-        <f>E27-D27</f>
-        <v/>
-      </c>
-      <c r="F35" s="20">
-        <f>F27-E27</f>
-        <v/>
-      </c>
+      <c r="A35" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   of which book publishers paid on consumption (change in C, negative)</t>
-        </is>
-      </c>
-      <c r="D36" s="20">
-        <f>-(D29-C29)</f>
-        <v/>
-      </c>
-      <c r="E36" s="20">
-        <f>-(E29-D29)</f>
-        <v/>
-      </c>
-      <c r="F36" s="20">
-        <f>-(F29-E29)</f>
-        <v/>
+      <c r="A36" s="17" t="inlineStr">
+        <is>
+          <t>d. Hand-back to direct-licensed publishers</t>
+        </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   of which paid hours (change in A)</t>
-        </is>
-      </c>
-      <c r="D37" s="20">
-        <f>D28-C28</f>
-        <v/>
-      </c>
-      <c r="E37" s="20">
-        <f>E28-D28</f>
-        <v/>
-      </c>
-      <c r="F37" s="20">
-        <f>F28-E28</f>
-        <v/>
+      <c r="A37" s="17" t="inlineStr">
+        <is>
+          <t>Publisher (share of US mechanicals in col B)</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="inlineStr">
+        <is>
+          <t>Months on direct licence</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Consensus gross-margin expansion, bp</t>
-        </is>
-      </c>
-      <c r="E38" s="24">
-        <f>Audiobooks_Inputs!$B$68</f>
-        <v/>
-      </c>
-      <c r="F38" s="24">
-        <f>Audiobooks_Inputs!$B$69</f>
-        <v/>
+          <t>UMPG</t>
+        </is>
+      </c>
+      <c r="B38" s="28">
+        <f>Audiobooks_Inputs!$B$49</f>
+        <v/>
+      </c>
+      <c r="C38" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" s="29">
+        <f>13-Audiobooks_Inputs!$B$54</f>
+        <v/>
+      </c>
+      <c r="E38" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F38" s="10" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Audiobook headwind as share of consensus expansion</t>
-        </is>
-      </c>
-      <c r="E39" s="25">
-        <f>-E34/E38</f>
-        <v/>
-      </c>
-      <c r="F39" s="25">
-        <f>-F34/F38</f>
-        <v/>
+          <t>Warner Chappell</t>
+        </is>
+      </c>
+      <c r="B39" s="28">
+        <f>Audiobooks_Inputs!$B$50</f>
+        <v/>
+      </c>
+      <c r="C39" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="29">
+        <f>13-Audiobooks_Inputs!$B$55</f>
+        <v/>
+      </c>
+      <c r="E39" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F39" s="10" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Memo (excluded from N): Jun-24 US price increase, annualized €M</t>
-        </is>
-      </c>
-      <c r="C40" s="19">
-        <f>Audiobooks_Inputs!$B$70</f>
-        <v/>
+          <t>Kobalt</t>
+        </is>
+      </c>
+      <c r="B40" s="28">
+        <f>Audiobooks_Inputs!$B$51</f>
+        <v/>
+      </c>
+      <c r="C40" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" s="29">
+        <f>13-Audiobooks_Inputs!$B$56</f>
+        <v/>
+      </c>
+      <c r="E40" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F40" s="10" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="41">
-      <c r="A41" t="inlineStr"/>
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Sony Music Publishing</t>
+        </is>
+      </c>
+      <c r="B41" s="28">
+        <f>Audiobooks_Inputs!$B$52</f>
+        <v/>
+      </c>
+      <c r="C41" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="29">
+        <f>13-Audiobooks_Inputs!$B$57</f>
+        <v/>
+      </c>
+      <c r="E41" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F41" s="10" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="42">
-      <c r="A42" s="16" t="inlineStr">
-        <is>
-          <t>5. Paid attach</t>
-        </is>
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>BMG</t>
+        </is>
+      </c>
+      <c r="B42" s="28">
+        <f>Audiobooks_Inputs!$B$53</f>
+        <v/>
+      </c>
+      <c r="C42" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" s="29">
+        <f>13-Audiobooks_Inputs!$B$58</f>
+        <v/>
+      </c>
+      <c r="E42" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="F42" s="10" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Audiobooks+ paying users (M)</t>
-        </is>
-      </c>
-      <c r="B43" s="26">
-        <f>Audiobooks_Inputs!$B$56</f>
+          <t>Sum of shares on direct licences (independents are the remainder, still paid at the bundle rate via the MLC)</t>
+        </is>
+      </c>
+      <c r="B43" s="30">
+        <f>SUM(B38:B42)</f>
         <v/>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ARR per payer ($ per year)</t>
-        </is>
-      </c>
-      <c r="B44" s="21">
-        <f>Audiobooks_Inputs!$B$55/Audiobooks_Inputs!$B$56</f>
+          <t>Restoration of the bundle discount in the direct deals</t>
+        </is>
+      </c>
+      <c r="B44" s="28">
+        <f>Audiobooks_Inputs!$B$59</f>
         <v/>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Payers / global Premium subscribers</t>
-        </is>
-      </c>
-      <c r="B45" s="27">
-        <f>$B$43/Audiobooks_Inputs!$B$62</f>
+          <t>Hand-back = gross x sum(share x months / 12) x restoration</t>
+        </is>
+      </c>
+      <c r="C45" s="22">
+        <f>C23*SUMPRODUCT($B$38:$B$42,C38:C42)/12*$B$44</f>
+        <v/>
+      </c>
+      <c r="D45" s="22">
+        <f>D23*SUMPRODUCT($B$38:$B$42,D38:D42)/12*$B$44</f>
+        <v/>
+      </c>
+      <c r="E45" s="22">
+        <f>E23*SUMPRODUCT($B$38:$B$42,E38:E42)/12*$B$44</f>
+        <v/>
+      </c>
+      <c r="F45" s="22">
+        <f>F23*SUMPRODUCT($B$38:$B$42,F38:F42)/12*$B$44</f>
         <v/>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="inlineStr">
-        <is>
-          <t>Payers / Premium subscribers in eligible markets</t>
-        </is>
-      </c>
-      <c r="B46" s="27">
-        <f>$B$43/Audiobooks_Inputs!$B$63</f>
+      <c r="A46" s="17" t="inlineStr">
+        <is>
+          <t>B  Net bundle saving (2027: if MLC switch = 1, the independents' share goes to zero)</t>
+        </is>
+      </c>
+      <c r="C46" s="22">
+        <f>C23-C45</f>
+        <v/>
+      </c>
+      <c r="D46" s="22">
+        <f>D23-D45</f>
+        <v/>
+      </c>
+      <c r="E46" s="22">
+        <f>E23-E45</f>
+        <v/>
+      </c>
+      <c r="F46" s="21">
+        <f>IF(Audiobooks_Inputs!$B$60=1,F23*$B$43*(1-$B$44),F23-F45)</f>
         <v/>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>Payers / monthly audiobook listeners, eligible markets</t>
-        </is>
-      </c>
-      <c r="B47" s="27">
-        <f>$B$43/(Audiobooks_Inputs!$B$63*Audiobooks_Inputs!$B$64)</f>
-        <v/>
-      </c>
+      <c r="A47" t="inlineStr"/>
     </row>
     <row r="48">
-      <c r="A48" t="inlineStr">
-        <is>
-          <t>Payers / monthly audiobook listeners, global</t>
-        </is>
-      </c>
-      <c r="B48" s="27">
-        <f>$B$43/(Audiobooks_Inputs!$B$62*Audiobooks_Inputs!$B$64)</f>
-        <v/>
+      <c r="A48" s="17" t="inlineStr">
+        <is>
+          <t>2. Audiobook licensing cost on included hours (C)</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Eligible Premium users who have ever pressed play</t>
-        </is>
-      </c>
-      <c r="B49" s="27">
-        <f>Audiobooks_Inputs!$B$65</f>
+          <t>Growth y/y</t>
+        </is>
+      </c>
+      <c r="D49" s="28">
+        <f>Audiobooks_Inputs!$B$62</f>
+        <v/>
+      </c>
+      <c r="E49" s="28">
+        <f>Audiobooks_Inputs!$B$63</f>
+        <v/>
+      </c>
+      <c r="F49" s="28">
+        <f>Audiobooks_Inputs!$B$64</f>
         <v/>
       </c>
     </row>
     <row r="50">
-      <c r="A50" t="inlineStr">
-        <is>
-          <t>US individual subscribers who took the $1 Basic plan (opt-out)</t>
-        </is>
-      </c>
-      <c r="B50" s="27">
-        <f>Audiobooks_Inputs!$B$66</f>
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>C  Base case</t>
+        </is>
+      </c>
+      <c r="C50" s="21">
+        <f>Audiobooks_Inputs!$B$61</f>
+        <v/>
+      </c>
+      <c r="D50" s="22">
+        <f>C50*(1+D49)</f>
+        <v/>
+      </c>
+      <c r="E50" s="22">
+        <f>D50*(1+E49)</f>
+        <v/>
+      </c>
+      <c r="F50" s="22">
+        <f>E50*(1+F49)</f>
         <v/>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Music Pro attach assumption, bull case</t>
-        </is>
-      </c>
-      <c r="B51" s="27">
-        <f>Audiobooks_Inputs!$B$67</f>
+          <t>C  Low case</t>
+        </is>
+      </c>
+      <c r="C51" s="21">
+        <f>C50*Audiobooks_Inputs!$B$65</f>
+        <v/>
+      </c>
+      <c r="D51" s="21">
+        <f>D50*Audiobooks_Inputs!$B$65</f>
+        <v/>
+      </c>
+      <c r="E51" s="21">
+        <f>E50*Audiobooks_Inputs!$B$65</f>
+        <v/>
+      </c>
+      <c r="F51" s="21">
+        <f>F50*Audiobooks_Inputs!$B$65</f>
         <v/>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr"/>
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>C  High case</t>
+        </is>
+      </c>
+      <c r="C52" s="21">
+        <f>C50*Audiobooks_Inputs!$B$66</f>
+        <v/>
+      </c>
+      <c r="D52" s="21">
+        <f>D50*Audiobooks_Inputs!$B$66</f>
+        <v/>
+      </c>
+      <c r="E52" s="21">
+        <f>E50*Audiobooks_Inputs!$B$66</f>
+        <v/>
+      </c>
+      <c r="F52" s="21">
+        <f>F50*Audiobooks_Inputs!$B$66</f>
+        <v/>
+      </c>
     </row>
     <row r="53">
-      <c r="A53" s="16" t="inlineStr">
-        <is>
-          <t>6. Cross-checks</t>
-        </is>
-      </c>
+      <c r="A53" t="inlineStr"/>
     </row>
     <row r="54">
-      <c r="A54" s="16" t="inlineStr">
-        <is>
-          <t>a. Market-share triangulation of C (2025)</t>
+      <c r="A54" s="17" t="inlineStr">
+        <is>
+          <t>3. Priced channel (Audiobooks+, top-ups, a la carte)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>US audiobook publisher receipts 2025 ($M)</t>
-        </is>
-      </c>
-      <c r="B55" s="19">
-        <f>Audiobooks_Inputs!$B$49</f>
+          <t>Revenue</t>
+        </is>
+      </c>
+      <c r="C55" s="21">
+        <f>Audiobooks_Inputs!$B$75</f>
+        <v/>
+      </c>
+      <c r="D55" s="21">
+        <f>Audiobooks_Inputs!$B$76</f>
+        <v/>
+      </c>
+      <c r="E55" s="21">
+        <f>Audiobooks_Inputs!$B$77</f>
+        <v/>
+      </c>
+      <c r="F55" s="21">
+        <f>Audiobooks_Inputs!$B$78</f>
         <v/>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Spotify share of US receipts: low (col B), high (col C)</t>
-        </is>
-      </c>
-      <c r="B56" s="22">
-        <f>Audiobooks_Inputs!$B$51</f>
-        <v/>
-      </c>
-      <c r="C56" s="22">
-        <f>Audiobooks_Inputs!$B$52</f>
+          <t>Content cost ratio on paid hours</t>
+        </is>
+      </c>
+      <c r="B56" s="28">
+        <f>Audiobooks_Inputs!$B$79</f>
         <v/>
       </c>
     </row>
     <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>Non-US markets, multiple of US cost</t>
-        </is>
-      </c>
-      <c r="B57" s="28">
-        <f>Audiobooks_Inputs!$B$53</f>
+      <c r="A57" s="17" t="inlineStr">
+        <is>
+          <t>A  Gross profit on paid hours = revenue x (1 - ratio)</t>
+        </is>
+      </c>
+      <c r="C57" s="22">
+        <f>C55*(1-$B$56)</f>
+        <v/>
+      </c>
+      <c r="D57" s="22">
+        <f>D55*(1-$B$56)</f>
+        <v/>
+      </c>
+      <c r="E57" s="22">
+        <f>E55*(1-$B$56)</f>
+        <v/>
+      </c>
+      <c r="F57" s="22">
+        <f>F55*(1-$B$56)</f>
         <v/>
       </c>
     </row>
     <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>EUR/USD</t>
-        </is>
-      </c>
-      <c r="B58" s="28">
-        <f>Audiobooks_Inputs!$B$54</f>
-        <v/>
-      </c>
+      <c r="A58" t="inlineStr"/>
     </row>
     <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>Implied global C 2025, €M: low (col B), high (col C)</t>
-        </is>
-      </c>
-      <c r="B59" s="20">
-        <f>B55*B56*B57/B58</f>
-        <v/>
-      </c>
-      <c r="C59" s="20">
-        <f>B55*C56*B57/B58</f>
-        <v/>
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>4. Net contribution to gross profit: N = B + A - C</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Base case C 2025, €M</t>
-        </is>
-      </c>
-      <c r="B60" s="20">
-        <f>D17</f>
+          <t>B  Net bundle saving</t>
+        </is>
+      </c>
+      <c r="C60" s="22">
+        <f>C46</f>
+        <v/>
+      </c>
+      <c r="D60" s="22">
+        <f>D46</f>
+        <v/>
+      </c>
+      <c r="E60" s="22">
+        <f>E46</f>
+        <v/>
+      </c>
+      <c r="F60" s="22">
+        <f>F46</f>
         <v/>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>Base case vs implied range: vs low (col B), vs high (col C)</t>
-        </is>
-      </c>
-      <c r="B61" s="29">
-        <f>B60/B59-1</f>
-        <v/>
-      </c>
-      <c r="C61" s="29">
-        <f>B60/C59-1</f>
+          <t>A  Gross profit on paid hours</t>
+        </is>
+      </c>
+      <c r="C61" s="22">
+        <f>C57</f>
+        <v/>
+      </c>
+      <c r="D61" s="22">
+        <f>D57</f>
+        <v/>
+      </c>
+      <c r="E61" s="22">
+        <f>E57</f>
+        <v/>
+      </c>
+      <c r="F61" s="22">
+        <f>F57</f>
         <v/>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="inlineStr"/>
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>C  Licensing cost on included hours</t>
+        </is>
+      </c>
+      <c r="C62" s="22">
+        <f>C50</f>
+        <v/>
+      </c>
+      <c r="D62" s="22">
+        <f>D50</f>
+        <v/>
+      </c>
+      <c r="E62" s="22">
+        <f>E50</f>
+        <v/>
+      </c>
+      <c r="F62" s="22">
+        <f>F50</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
-      <c r="A63" s="16" t="inlineStr">
-        <is>
-          <t>b. Incremental Premium content-cost ratio (does the P&amp;L show an audiobook step?)</t>
-        </is>
+      <c r="A63" s="17" t="inlineStr">
+        <is>
+          <t>N  Net contribution</t>
+        </is>
+      </c>
+      <c r="C63" s="22">
+        <f>C60+C61-C62</f>
+        <v/>
+      </c>
+      <c r="D63" s="22">
+        <f>D60+D61-D62</f>
+        <v/>
+      </c>
+      <c r="E63" s="22">
+        <f>E60+E61-E62</f>
+        <v/>
+      </c>
+      <c r="F63" s="22">
+        <f>F60+F61-F62</f>
+        <v/>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="16" t="inlineStr"/>
-      <c r="C64" s="30" t="inlineStr">
-        <is>
-          <t>Premium revenue change</t>
-        </is>
-      </c>
-      <c r="D64" s="30" t="inlineStr">
-        <is>
-          <t>Content cost change</t>
-        </is>
-      </c>
-      <c r="E64" s="30" t="inlineStr">
-        <is>
-          <t>Incremental ratio</t>
-        </is>
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Group revenue</t>
+        </is>
+      </c>
+      <c r="C64" s="21">
+        <f>Audiobooks_Inputs!$B$12</f>
+        <v/>
+      </c>
+      <c r="D64" s="21">
+        <f>Audiobooks_Inputs!$B$13</f>
+        <v/>
+      </c>
+      <c r="E64" s="21">
+        <f>Audiobooks_Inputs!$B$14</f>
+        <v/>
+      </c>
+      <c r="F64" s="21">
+        <f>Audiobooks_Inputs!$B$15</f>
+        <v/>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FY24 vs FY23</t>
-        </is>
-      </c>
-      <c r="C65" s="19">
-        <f>Audiobooks_Inputs!$B$7-Audiobooks_Inputs!$B$6</f>
-        <v/>
-      </c>
-      <c r="D65" s="19">
-        <f>Audiobooks_Inputs!$B$21</f>
-        <v/>
-      </c>
-      <c r="E65" s="29">
-        <f>D65/C65</f>
+          <t>N, bp of group revenue</t>
+        </is>
+      </c>
+      <c r="C65" s="31">
+        <f>C63/C64*10000</f>
+        <v/>
+      </c>
+      <c r="D65" s="31">
+        <f>D63/D64*10000</f>
+        <v/>
+      </c>
+      <c r="E65" s="31">
+        <f>E63/E64*10000</f>
+        <v/>
+      </c>
+      <c r="F65" s="31">
+        <f>F63/F64*10000</f>
         <v/>
       </c>
     </row>
     <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>FY25 vs FY24</t>
-        </is>
-      </c>
-      <c r="C66" s="19">
-        <f>Audiobooks_Inputs!$B$8-Audiobooks_Inputs!$B$7</f>
-        <v/>
-      </c>
-      <c r="D66" s="19">
-        <f>Audiobooks_Inputs!$B$22</f>
-        <v/>
-      </c>
-      <c r="E66" s="29">
-        <f>D66/C66</f>
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>Change in N y/y, €M (gross-margin headwind)</t>
+        </is>
+      </c>
+      <c r="D66" s="22">
+        <f>D63-C63</f>
+        <v/>
+      </c>
+      <c r="E66" s="22">
+        <f>E63-D63</f>
+        <v/>
+      </c>
+      <c r="F66" s="22">
+        <f>F63-E63</f>
         <v/>
       </c>
     </row>
     <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>9M-25 vs 9M-24</t>
-        </is>
-      </c>
-      <c r="C67" s="19">
-        <f>Audiobooks_Inputs!$B$28-Audiobooks_Inputs!$B$27</f>
-        <v/>
-      </c>
-      <c r="D67" s="19">
-        <f>Audiobooks_Inputs!$B$23</f>
-        <v/>
-      </c>
-      <c r="E67" s="29">
-        <f>D67/C67</f>
+      <c r="A67" s="17" t="inlineStr">
+        <is>
+          <t>Change in N y/y, bp of group revenue</t>
+        </is>
+      </c>
+      <c r="D67" s="31">
+        <f>D66/D64*10000</f>
+        <v/>
+      </c>
+      <c r="E67" s="31">
+        <f>E66/E64*10000</f>
+        <v/>
+      </c>
+      <c r="F67" s="31">
+        <f>F66/F64*10000</f>
         <v/>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>H1-26 vs H1-25</t>
-        </is>
-      </c>
-      <c r="C68" s="19">
-        <f>Audiobooks_Inputs!$B$26-Audiobooks_Inputs!$B$25</f>
-        <v/>
-      </c>
-      <c r="D68" s="19">
-        <f>Audiobooks_Inputs!$B$24</f>
-        <v/>
-      </c>
-      <c r="E68" s="29">
-        <f>D68/C68</f>
+          <t xml:space="preserve">   of which music publishers reclaim the bundle saving (change in B)</t>
+        </is>
+      </c>
+      <c r="D68" s="22">
+        <f>D60-C60</f>
+        <v/>
+      </c>
+      <c r="E68" s="22">
+        <f>E60-D60</f>
+        <v/>
+      </c>
+      <c r="F68" s="22">
+        <f>F60-E60</f>
         <v/>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Note: the incremental ratio holds at 48-50% in every period against a ~66% average ratio. It bounds the growth in C rather than measuring it: music royalties, the bundle saving, marketplace offsets and the Partner Program all move inside the same line.</t>
-        </is>
+          <t xml:space="preserve">   of which book publishers paid on consumption (change in C, negative)</t>
+        </is>
+      </c>
+      <c r="D69" s="22">
+        <f>-(D62-C62)</f>
+        <v/>
+      </c>
+      <c r="E69" s="22">
+        <f>-(E62-D62)</f>
+        <v/>
+      </c>
+      <c r="F69" s="22">
+        <f>-(F62-E62)</f>
+        <v/>
       </c>
     </row>
     <row r="70">
-      <c r="A70" t="inlineStr"/>
+      <c r="A70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   of which paid hours (change in A)</t>
+        </is>
+      </c>
+      <c r="D70" s="22">
+        <f>D61-C61</f>
+        <v/>
+      </c>
+      <c r="E70" s="22">
+        <f>E61-D61</f>
+        <v/>
+      </c>
+      <c r="F70" s="22">
+        <f>F61-E61</f>
+        <v/>
+      </c>
     </row>
     <row r="71">
-      <c r="A71" s="16" t="inlineStr">
-        <is>
-          <t>c. Bundle saving, external references</t>
-        </is>
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Consensus gross-margin expansion, bp</t>
+        </is>
+      </c>
+      <c r="E71" s="32">
+        <f>Audiobooks_Inputs!$B$86</f>
+        <v/>
+      </c>
+      <c r="F71" s="32">
+        <f>Audiobooks_Inputs!$B$87</f>
+        <v/>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>NMPA first-year publisher loss estimate ($M)</t>
-        </is>
-      </c>
-      <c r="B72" s="19">
-        <f>Audiobooks_Inputs!$B$31</f>
+          <t>Audiobook headwind as share of consensus expansion</t>
+        </is>
+      </c>
+      <c r="E72" s="30">
+        <f>-E67/E71</f>
+        <v/>
+      </c>
+      <c r="F72" s="30">
+        <f>-F67/F71</f>
         <v/>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>MLC mechanical royalties paid, $M: Q4-23 (col B), Q4-25 (col C); direct-licensed publishers leave the MLC pool after 2025, so the series overstates the net saving</t>
-        </is>
-      </c>
-      <c r="B73" s="26">
-        <f>Audiobooks_Inputs!$B$32</f>
-        <v/>
-      </c>
-      <c r="C73" s="26">
-        <f>Audiobooks_Inputs!$B$33</f>
+          <t>Memo (excluded from N): Jun-24 US price increase, annualized €M</t>
+        </is>
+      </c>
+      <c r="C73" s="21">
+        <f>Audiobooks_Inputs!$B$88</f>
         <v/>
       </c>
     </row>
@@ -3648,228 +4321,554 @@
       <c r="A74" t="inlineStr"/>
     </row>
     <row r="75">
-      <c r="A75" s="16" t="inlineStr">
-        <is>
-          <t>7. Sensitivity: 2027E, by audiobook cost growth (rows) and bundle-discount restoration / MLC outcome (columns)</t>
+      <c r="A75" s="17" t="inlineStr">
+        <is>
+          <t>5. Paid attach</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Restoration of bundle discount</t>
-        </is>
-      </c>
-      <c r="C76" s="31" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D76" s="31" t="n">
-        <v>1</v>
-      </c>
-      <c r="E76" s="31" t="n">
-        <v>1</v>
+          <t>Audiobooks+ paying users (M)</t>
+        </is>
+      </c>
+      <c r="B76" s="24">
+        <f>Audiobooks_Inputs!$B$74</f>
+        <v/>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>MLC complaint succeeds in 2027 (1 = yes)</t>
-        </is>
-      </c>
-      <c r="C77" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="D77" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="E77" s="7" t="n">
-        <v>1</v>
+          <t>ARR per payer ($ per year)</t>
+        </is>
+      </c>
+      <c r="B77" s="29">
+        <f>Audiobooks_Inputs!$B$73/Audiobooks_Inputs!$B$74</f>
+        <v/>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="16" t="inlineStr">
-        <is>
-          <t>Cost growth p.a. 2026-27 (col A)</t>
-        </is>
-      </c>
-      <c r="C78" s="30" t="inlineStr">
-        <is>
-          <t>Change in N 2027, bp</t>
-        </is>
-      </c>
-      <c r="D78" s="30" t="inlineStr">
-        <is>
-          <t>Change in N 2027, bp</t>
-        </is>
-      </c>
-      <c r="E78" s="30" t="inlineStr">
-        <is>
-          <t>Change in N 2027, bp</t>
-        </is>
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Payers / global Premium subscribers</t>
+        </is>
+      </c>
+      <c r="B78" s="33">
+        <f>$B$76/Audiobooks_Inputs!$B$80</f>
+        <v/>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="31" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C79" s="24">
-        <f>((IF(C$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))+($F$24-$E$24)-$D$17*(1+$A79)*$A79)/$F$31*10000</f>
-        <v/>
-      </c>
-      <c r="D79" s="24">
-        <f>((IF(D$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))+($F$24-$E$24)-$D$17*(1+$A79)*$A79)/$F$31*10000</f>
-        <v/>
-      </c>
-      <c r="E79" s="24">
-        <f>((IF(E$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))+($F$24-$E$24)-$D$17*(1+$A79)*$A79)/$F$31*10000</f>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Payers / Premium subscribers in eligible markets</t>
+        </is>
+      </c>
+      <c r="B79" s="33">
+        <f>$B$76/Audiobooks_Inputs!$B$81</f>
         <v/>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="31" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C80" s="24">
-        <f>((IF(C$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))+($F$24-$E$24)-$D$17*(1+$A80)*$A80)/$F$31*10000</f>
-        <v/>
-      </c>
-      <c r="D80" s="24">
-        <f>((IF(D$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))+($F$24-$E$24)-$D$17*(1+$A80)*$A80)/$F$31*10000</f>
-        <v/>
-      </c>
-      <c r="E80" s="24">
-        <f>((IF(E$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))+($F$24-$E$24)-$D$17*(1+$A80)*$A80)/$F$31*10000</f>
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Payers / monthly audiobook listeners, eligible markets</t>
+        </is>
+      </c>
+      <c r="B80" s="33">
+        <f>$B$76/(Audiobooks_Inputs!$B$81*Audiobooks_Inputs!$B$82)</f>
         <v/>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="31" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="C81" s="24">
-        <f>((IF(C$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))+($F$24-$E$24)-$D$17*(1+$A81)*$A81)/$F$31*10000</f>
-        <v/>
-      </c>
-      <c r="D81" s="24">
-        <f>((IF(D$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))+($F$24-$E$24)-$D$17*(1+$A81)*$A81)/$F$31*10000</f>
-        <v/>
-      </c>
-      <c r="E81" s="24">
-        <f>((IF(E$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))+($F$24-$E$24)-$D$17*(1+$A81)*$A81)/$F$31*10000</f>
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Payers / monthly audiobook listeners, global</t>
+        </is>
+      </c>
+      <c r="B81" s="33">
+        <f>$B$76/(Audiobooks_Inputs!$B$80*Audiobooks_Inputs!$B$82)</f>
         <v/>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="31" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C82" s="24">
-        <f>((IF(C$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))+($F$24-$E$24)-$D$17*(1+$A82)*$A82)/$F$31*10000</f>
-        <v/>
-      </c>
-      <c r="D82" s="24">
-        <f>((IF(D$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))+($F$24-$E$24)-$D$17*(1+$A82)*$A82)/$F$31*10000</f>
-        <v/>
-      </c>
-      <c r="E82" s="24">
-        <f>((IF(E$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))-$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))+($F$24-$E$24)-$D$17*(1+$A82)*$A82)/$F$31*10000</f>
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Eligible Premium users who have ever pressed play</t>
+        </is>
+      </c>
+      <c r="B82" s="33">
+        <f>Audiobooks_Inputs!$B$83</f>
         <v/>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="16" t="inlineStr">
-        <is>
-          <t>Cost growth p.a. 2026-27 (col A)</t>
-        </is>
-      </c>
-      <c r="C83" s="30" t="inlineStr">
-        <is>
-          <t>N 2027, €M</t>
-        </is>
-      </c>
-      <c r="D83" s="30" t="inlineStr">
-        <is>
-          <t>N 2027, €M</t>
-        </is>
-      </c>
-      <c r="E83" s="30" t="inlineStr">
-        <is>
-          <t>N 2027, €M</t>
-        </is>
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>US individual subscribers who took the $1 Basic plan (opt-out)</t>
+        </is>
+      </c>
+      <c r="B83" s="33">
+        <f>Audiobooks_Inputs!$B$84</f>
+        <v/>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="31" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C84" s="19">
-        <f>IF(C$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))+$F$24-$D$17*(1+$A84)^2</f>
-        <v/>
-      </c>
-      <c r="D84" s="19">
-        <f>IF(D$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))+$F$24-$D$17*(1+$A84)^2</f>
-        <v/>
-      </c>
-      <c r="E84" s="19">
-        <f>IF(E$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))+$F$24-$D$17*(1+$A84)^2</f>
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Music Pro attach assumption, bull case</t>
+        </is>
+      </c>
+      <c r="B84" s="33">
+        <f>Audiobooks_Inputs!$B$85</f>
         <v/>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="31" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="C85" s="19">
-        <f>IF(C$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))+$F$24-$D$17*(1+$A85)^2</f>
-        <v/>
-      </c>
-      <c r="D85" s="19">
-        <f>IF(D$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))+$F$24-$D$17*(1+$A85)^2</f>
-        <v/>
-      </c>
-      <c r="E85" s="19">
-        <f>IF(E$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))+$F$24-$D$17*(1+$A85)^2</f>
-        <v/>
-      </c>
+      <c r="A85" t="inlineStr"/>
     </row>
     <row r="86">
-      <c r="A86" s="31" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="C86" s="19">
-        <f>IF(C$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))+$F$24-$D$17*(1+$A86)^2</f>
-        <v/>
-      </c>
-      <c r="D86" s="19">
-        <f>IF(D$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))+$F$24-$D$17*(1+$A86)^2</f>
-        <v/>
-      </c>
-      <c r="E86" s="19">
-        <f>IF(E$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))+$F$24-$D$17*(1+$A86)^2</f>
-        <v/>
+      <c r="A86" s="17" t="inlineStr">
+        <is>
+          <t>6. Cross-checks</t>
+        </is>
       </c>
     </row>
     <row r="87">
-      <c r="A87" s="31" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="C87" s="19">
-        <f>IF(C$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*C$76))+$F$24-$D$17*(1+$A87)^2</f>
-        <v/>
-      </c>
-      <c r="D87" s="19">
-        <f>IF(D$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*D$76))+$F$24-$D$17*(1+$A87)^2</f>
-        <v/>
-      </c>
-      <c r="E87" s="19">
-        <f>IF(E$77=1,0,$B$6*(1-(Audiobooks_Inputs!$B$35+Audiobooks_Inputs!$B$36+Audiobooks_Inputs!$B$37)*E$76))+$F$24-$D$17*(1+$A87)^2</f>
-        <v/>
+      <c r="A87" s="17" t="inlineStr">
+        <is>
+          <t>a. Market-share triangulation of C (2025)</t>
+        </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Restoration below 100% does not change the 2027 headwind (B is flat 2026 to 2027 once all three majors are on direct licences); it changes the level of N.</t>
+          <t>US audiobook publisher receipts 2025 ($M)</t>
+        </is>
+      </c>
+      <c r="B88" s="21">
+        <f>Audiobooks_Inputs!$B$67</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Spotify share of US receipts: low (col B), high (col C)</t>
+        </is>
+      </c>
+      <c r="B89" s="28">
+        <f>Audiobooks_Inputs!$B$69</f>
+        <v/>
+      </c>
+      <c r="C89" s="28">
+        <f>Audiobooks_Inputs!$B$70</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Non-US markets, multiple of US cost</t>
+        </is>
+      </c>
+      <c r="B90" s="26">
+        <f>Audiobooks_Inputs!$B$71</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>EUR/USD</t>
+        </is>
+      </c>
+      <c r="B91" s="26">
+        <f>Audiobooks_Inputs!$B$72</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Implied global C 2025, €M: low (col B), high (col C)</t>
+        </is>
+      </c>
+      <c r="B92" s="22">
+        <f>B88*B89*B90/B91</f>
+        <v/>
+      </c>
+      <c r="C92" s="22">
+        <f>B88*C89*B90/B91</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Base case C 2025, €M</t>
+        </is>
+      </c>
+      <c r="B93" s="22">
+        <f>D50</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Base case vs implied range: vs low (col B), vs high (col C)</t>
+        </is>
+      </c>
+      <c r="B94" s="34">
+        <f>B93/B92-1</f>
+        <v/>
+      </c>
+      <c r="C94" s="34">
+        <f>B93/C92-1</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="17" t="inlineStr">
+        <is>
+          <t>b. Incremental Premium content-cost ratio (does the P&amp;L show an audiobook step?)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="17" t="inlineStr"/>
+      <c r="C97" s="20" t="inlineStr">
+        <is>
+          <t>Premium revenue change</t>
+        </is>
+      </c>
+      <c r="D97" s="20" t="inlineStr">
+        <is>
+          <t>Content cost change</t>
+        </is>
+      </c>
+      <c r="E97" s="20" t="inlineStr">
+        <is>
+          <t>Incremental ratio</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>FY24 vs FY23</t>
+        </is>
+      </c>
+      <c r="C98" s="21">
+        <f>Audiobooks_Inputs!$B$7-Audiobooks_Inputs!$B$6</f>
+        <v/>
+      </c>
+      <c r="D98" s="21">
+        <f>Audiobooks_Inputs!$B$21</f>
+        <v/>
+      </c>
+      <c r="E98" s="34">
+        <f>D98/C98</f>
+        <v/>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>FY25 vs FY24</t>
+        </is>
+      </c>
+      <c r="C99" s="21">
+        <f>Audiobooks_Inputs!$B$8-Audiobooks_Inputs!$B$7</f>
+        <v/>
+      </c>
+      <c r="D99" s="21">
+        <f>Audiobooks_Inputs!$B$22</f>
+        <v/>
+      </c>
+      <c r="E99" s="34">
+        <f>D99/C99</f>
+        <v/>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>9M-25 vs 9M-24</t>
+        </is>
+      </c>
+      <c r="C100" s="21">
+        <f>Audiobooks_Inputs!$B$28-Audiobooks_Inputs!$B$27</f>
+        <v/>
+      </c>
+      <c r="D100" s="21">
+        <f>Audiobooks_Inputs!$B$23</f>
+        <v/>
+      </c>
+      <c r="E100" s="34">
+        <f>D100/C100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>H1-26 vs H1-25</t>
+        </is>
+      </c>
+      <c r="C101" s="21">
+        <f>Audiobooks_Inputs!$B$26-Audiobooks_Inputs!$B$25</f>
+        <v/>
+      </c>
+      <c r="D101" s="21">
+        <f>Audiobooks_Inputs!$B$24</f>
+        <v/>
+      </c>
+      <c r="E101" s="34">
+        <f>D101/C101</f>
+        <v/>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Note: the incremental ratio holds at 48-50% in every period against a ~66% average ratio. It bounds the growth in C rather than measuring it: music royalties, the bundle saving, marketplace offsets and the Partner Program all move inside the same line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="17" t="inlineStr">
+        <is>
+          <t>7. Sensitivity: 2027E, by audiobook cost growth (rows) and bundle-discount restoration / MLC outcome (columns)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Restoration of bundle discount</t>
+        </is>
+      </c>
+      <c r="C105" s="35" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="D105" s="35" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E105" s="35" t="n">
+        <v>0.75</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>MLC complaint succeeds in 2027 (1 = yes)</t>
+        </is>
+      </c>
+      <c r="C106" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D106" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="E106" s="10" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="17" t="inlineStr">
+        <is>
+          <t>Cost growth p.a. 2026-27 (col A)</t>
+        </is>
+      </c>
+      <c r="C107" s="20" t="inlineStr">
+        <is>
+          <t>Change in N 2027, bp</t>
+        </is>
+      </c>
+      <c r="D107" s="20" t="inlineStr">
+        <is>
+          <t>Change in N 2027, bp</t>
+        </is>
+      </c>
+      <c r="E107" s="20" t="inlineStr">
+        <is>
+          <t>Change in N 2027, bp</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="35" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C108" s="31">
+        <f>((IF(C$106=1,$F$23*$B$43*(1-C$105),$F$23*(1-$B$43*C$105))-$E$23*(1-$B$43*C$105))+($F$57-$E$57)-$D$50*(1+$A108)*$A108)/$F$64*10000</f>
+        <v/>
+      </c>
+      <c r="D108" s="31">
+        <f>((IF(D$106=1,$F$23*$B$43*(1-D$105),$F$23*(1-$B$43*D$105))-$E$23*(1-$B$43*D$105))+($F$57-$E$57)-$D$50*(1+$A108)*$A108)/$F$64*10000</f>
+        <v/>
+      </c>
+      <c r="E108" s="31">
+        <f>((IF(E$106=1,$F$23*$B$43*(1-E$105),$F$23*(1-$B$43*E$105))-$E$23*(1-$B$43*E$105))+($F$57-$E$57)-$D$50*(1+$A108)*$A108)/$F$64*10000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="35" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C109" s="31">
+        <f>((IF(C$106=1,$F$23*$B$43*(1-C$105),$F$23*(1-$B$43*C$105))-$E$23*(1-$B$43*C$105))+($F$57-$E$57)-$D$50*(1+$A109)*$A109)/$F$64*10000</f>
+        <v/>
+      </c>
+      <c r="D109" s="31">
+        <f>((IF(D$106=1,$F$23*$B$43*(1-D$105),$F$23*(1-$B$43*D$105))-$E$23*(1-$B$43*D$105))+($F$57-$E$57)-$D$50*(1+$A109)*$A109)/$F$64*10000</f>
+        <v/>
+      </c>
+      <c r="E109" s="31">
+        <f>((IF(E$106=1,$F$23*$B$43*(1-E$105),$F$23*(1-$B$43*E$105))-$E$23*(1-$B$43*E$105))+($F$57-$E$57)-$D$50*(1+$A109)*$A109)/$F$64*10000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="35" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C110" s="31">
+        <f>((IF(C$106=1,$F$23*$B$43*(1-C$105),$F$23*(1-$B$43*C$105))-$E$23*(1-$B$43*C$105))+($F$57-$E$57)-$D$50*(1+$A110)*$A110)/$F$64*10000</f>
+        <v/>
+      </c>
+      <c r="D110" s="31">
+        <f>((IF(D$106=1,$F$23*$B$43*(1-D$105),$F$23*(1-$B$43*D$105))-$E$23*(1-$B$43*D$105))+($F$57-$E$57)-$D$50*(1+$A110)*$A110)/$F$64*10000</f>
+        <v/>
+      </c>
+      <c r="E110" s="31">
+        <f>((IF(E$106=1,$F$23*$B$43*(1-E$105),$F$23*(1-$B$43*E$105))-$E$23*(1-$B$43*E$105))+($F$57-$E$57)-$D$50*(1+$A110)*$A110)/$F$64*10000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="35" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C111" s="31">
+        <f>((IF(C$106=1,$F$23*$B$43*(1-C$105),$F$23*(1-$B$43*C$105))-$E$23*(1-$B$43*C$105))+($F$57-$E$57)-$D$50*(1+$A111)*$A111)/$F$64*10000</f>
+        <v/>
+      </c>
+      <c r="D111" s="31">
+        <f>((IF(D$106=1,$F$23*$B$43*(1-D$105),$F$23*(1-$B$43*D$105))-$E$23*(1-$B$43*D$105))+($F$57-$E$57)-$D$50*(1+$A111)*$A111)/$F$64*10000</f>
+        <v/>
+      </c>
+      <c r="E111" s="31">
+        <f>((IF(E$106=1,$F$23*$B$43*(1-E$105),$F$23*(1-$B$43*E$105))-$E$23*(1-$B$43*E$105))+($F$57-$E$57)-$D$50*(1+$A111)*$A111)/$F$64*10000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="17" t="inlineStr">
+        <is>
+          <t>Cost growth p.a. 2026-27 (col A)</t>
+        </is>
+      </c>
+      <c r="C112" s="20" t="inlineStr">
+        <is>
+          <t>N 2027, €M</t>
+        </is>
+      </c>
+      <c r="D112" s="20" t="inlineStr">
+        <is>
+          <t>N 2027, €M</t>
+        </is>
+      </c>
+      <c r="E112" s="20" t="inlineStr">
+        <is>
+          <t>N 2027, €M</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="35" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C113" s="22">
+        <f>IF(C$106=1,$F$23*$B$43*(1-C$105),$F$23*(1-$B$43*C$105))+$F$57-$D$50*(1+$A113)^2</f>
+        <v/>
+      </c>
+      <c r="D113" s="22">
+        <f>IF(D$106=1,$F$23*$B$43*(1-D$105),$F$23*(1-$B$43*D$105))+$F$57-$D$50*(1+$A113)^2</f>
+        <v/>
+      </c>
+      <c r="E113" s="22">
+        <f>IF(E$106=1,$F$23*$B$43*(1-E$105),$F$23*(1-$B$43*E$105))+$F$57-$D$50*(1+$A113)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="35" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="C114" s="22">
+        <f>IF(C$106=1,$F$23*$B$43*(1-C$105),$F$23*(1-$B$43*C$105))+$F$57-$D$50*(1+$A114)^2</f>
+        <v/>
+      </c>
+      <c r="D114" s="22">
+        <f>IF(D$106=1,$F$23*$B$43*(1-D$105),$F$23*(1-$B$43*D$105))+$F$57-$D$50*(1+$A114)^2</f>
+        <v/>
+      </c>
+      <c r="E114" s="22">
+        <f>IF(E$106=1,$F$23*$B$43*(1-E$105),$F$23*(1-$B$43*E$105))+$F$57-$D$50*(1+$A114)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="35" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C115" s="22">
+        <f>IF(C$106=1,$F$23*$B$43*(1-C$105),$F$23*(1-$B$43*C$105))+$F$57-$D$50*(1+$A115)^2</f>
+        <v/>
+      </c>
+      <c r="D115" s="22">
+        <f>IF(D$106=1,$F$23*$B$43*(1-D$105),$F$23*(1-$B$43*D$105))+$F$57-$D$50*(1+$A115)^2</f>
+        <v/>
+      </c>
+      <c r="E115" s="22">
+        <f>IF(E$106=1,$F$23*$B$43*(1-E$105),$F$23*(1-$B$43*E$105))+$F$57-$D$50*(1+$A115)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="35" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C116" s="22">
+        <f>IF(C$106=1,$F$23*$B$43*(1-C$105),$F$23*(1-$B$43*C$105))+$F$57-$D$50*(1+$A116)^2</f>
+        <v/>
+      </c>
+      <c r="D116" s="22">
+        <f>IF(D$106=1,$F$23*$B$43*(1-D$105),$F$23*(1-$B$43*D$105))+$F$57-$D$50*(1+$A116)^2</f>
+        <v/>
+      </c>
+      <c r="E116" s="22">
+        <f>IF(E$106=1,$F$23*$B$43*(1-E$105),$F$23*(1-$B$43*E$105))+$F$57-$D$50*(1+$A116)^2</f>
+        <v/>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Restoration does not change the 2027 headwind (B is flat 2026 to 2027 once every direct deal is a full year old); it changes the level of N. An MLC win removes the independents' share of the gross saving.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Embed cached values in the audiobooks workbook; one-table cost-growth sensitivity
- Write each formula's computed value into the file so previews and
  viewers that do not recalculate show numbers; formulas stay live
- AB_Sensitivity reduced to a single table: licensing-cost growth
  applied to 2026E and 2027E against C, contribution and headwind,
  with the bridge base case shown underneath

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012Bq554HW2LcX3ZmUaAuu9U
</commit_message>
<xml_diff>
--- a/data/SPOT_audiobooks_model.xlsx
+++ b/data/SPOT_audiobooks_model.xlsx
@@ -24,7 +24,7 @@
     <numFmt numFmtId="166" formatCode="0.0"/>
     <numFmt numFmtId="167" formatCode="0_);(0)"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -54,10 +54,6 @@
     </font>
     <font>
       <i val="1"/>
-    </font>
-    <font>
-      <b val="1"/>
-      <color rgb="000000FF"/>
     </font>
   </fonts>
   <fills count="7">
@@ -105,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,11 +144,12 @@
     <xf numFmtId="37" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="6" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="167" fontId="5" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2241,18 +2238,18 @@
       </c>
       <c r="C7" s="20">
         <f>AB_Inputs!$B$12</f>
-        <v/>
+        <v>46.0</v>
       </c>
       <c r="D7" s="21">
         <f>C7</f>
-        <v/>
+        <v>46.0</v>
       </c>
       <c r="E7" s="5" t="n">
         <v>4</v>
       </c>
       <c r="F7" s="22">
         <f>D7/E7</f>
-        <v/>
+        <v>11.5</v>
       </c>
     </row>
     <row r="8">
@@ -2263,18 +2260,18 @@
       </c>
       <c r="C8" s="20">
         <f>AB_Inputs!$B$14</f>
-        <v/>
+        <v>94.0</v>
       </c>
       <c r="D8" s="21">
         <f>C8-C7</f>
-        <v/>
+        <v>48.0</v>
       </c>
       <c r="E8" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F8" s="22">
         <f>D8/E8</f>
-        <v/>
+        <v>16.0</v>
       </c>
     </row>
     <row r="9">
@@ -2285,18 +2282,18 @@
       </c>
       <c r="C9" s="20">
         <f>AB_Inputs!$B$15</f>
-        <v/>
+        <v>150.0</v>
       </c>
       <c r="D9" s="21">
         <f>C9-C8</f>
-        <v/>
+        <v>56.0</v>
       </c>
       <c r="E9" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F9" s="22">
         <f>D9/E9</f>
-        <v/>
+        <v>18.666666666666668</v>
       </c>
     </row>
     <row r="10">
@@ -2307,18 +2304,18 @@
       </c>
       <c r="C10" s="20">
         <f>AB_Inputs!$B$16</f>
-        <v/>
+        <v>205.0</v>
       </c>
       <c r="D10" s="21">
         <f>C10-C9</f>
-        <v/>
+        <v>55.0</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F10" s="22">
         <f>D10/E10</f>
-        <v/>
+        <v>18.333333333333332</v>
       </c>
     </row>
     <row r="11">
@@ -2329,18 +2326,18 @@
       </c>
       <c r="C11" s="20">
         <f>AB_Inputs!$B$17</f>
-        <v/>
+        <v>256.0</v>
       </c>
       <c r="D11" s="21">
         <f>C11-C10</f>
-        <v/>
+        <v>51.0</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F11" s="22">
         <f>D11/E11</f>
-        <v/>
+        <v>17.0</v>
       </c>
     </row>
     <row r="12">
@@ -2351,18 +2348,18 @@
       </c>
       <c r="C12" s="20">
         <f>AB_Inputs!$B$18</f>
-        <v/>
+        <v>308.0</v>
       </c>
       <c r="D12" s="21">
         <f>C12-C11</f>
-        <v/>
+        <v>52.0</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F12" s="22">
         <f>D12/E12</f>
-        <v/>
+        <v>17.333333333333332</v>
       </c>
     </row>
     <row r="13">
@@ -2373,18 +2370,18 @@
       </c>
       <c r="C13" s="20">
         <f>AB_Inputs!$B$19</f>
-        <v/>
+        <v>358.0</v>
       </c>
       <c r="D13" s="21">
         <f>C13-C12</f>
-        <v/>
+        <v>50.0</v>
       </c>
       <c r="E13" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F13" s="22">
         <f>D13/E13</f>
-        <v/>
+        <v>16.666666666666668</v>
       </c>
     </row>
     <row r="14">
@@ -2395,18 +2392,18 @@
       </c>
       <c r="C14" s="20">
         <f>AB_Inputs!$B$20</f>
-        <v/>
+        <v>410.0</v>
       </c>
       <c r="D14" s="21">
         <f>C14-C13</f>
-        <v/>
+        <v>52.0</v>
       </c>
       <c r="E14" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F14" s="22">
         <f>D14/E14</f>
-        <v/>
+        <v>17.333333333333332</v>
       </c>
     </row>
     <row r="15">
@@ -2417,18 +2414,18 @@
       </c>
       <c r="C15" s="20">
         <f>AB_Inputs!$B$21</f>
-        <v/>
+        <v>437.0</v>
       </c>
       <c r="D15" s="21">
         <f>C15-C14</f>
-        <v/>
+        <v>27.0</v>
       </c>
       <c r="E15" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F15" s="22">
         <f>D15/E15</f>
-        <v/>
+        <v>9.0</v>
       </c>
     </row>
     <row r="16">
@@ -2439,14 +2436,14 @@
       </c>
       <c r="C16" s="20">
         <f>AB_Inputs!$B$13</f>
-        <v/>
+        <v>35.0</v>
       </c>
       <c r="E16" s="5" t="n">
         <v>3</v>
       </c>
       <c r="F16" s="22">
         <f>C16/E16</f>
-        <v/>
+        <v>11.666666666666666</v>
       </c>
     </row>
     <row r="17">
@@ -2457,11 +2454,11 @@
       </c>
       <c r="B17" s="22">
         <f>AVERAGE(D11:D14)</f>
-        <v/>
+        <v>51.25</v>
       </c>
       <c r="C17" s="22">
         <f>B17*4</f>
-        <v/>
+        <v>205.0</v>
       </c>
     </row>
     <row r="18">
@@ -2489,11 +2486,11 @@
       </c>
       <c r="B21" s="23">
         <f>AB_Inputs!$B$26</f>
-        <v/>
+        <v>97.3</v>
       </c>
       <c r="C21" s="23">
         <f>AB_Inputs!$B$27</f>
-        <v/>
+        <v>53.3</v>
       </c>
     </row>
     <row r="22">
@@ -2504,11 +2501,11 @@
       </c>
       <c r="B22" s="24">
         <f>AB_Inputs!$B$28</f>
-        <v/>
+        <v>0.00068</v>
       </c>
       <c r="C22" s="24">
         <f>AB_Inputs!$B$29</f>
-        <v/>
+        <v>0.00033</v>
       </c>
     </row>
     <row r="23">
@@ -2519,11 +2516,11 @@
       </c>
       <c r="B23" s="22">
         <f>B21/B22/1000</f>
-        <v/>
+        <v>143.08823529411762</v>
       </c>
       <c r="C23" s="22">
         <f>C21/C22/1000</f>
-        <v/>
+        <v>161.51515151515153</v>
       </c>
     </row>
     <row r="24">
@@ -2534,7 +2531,7 @@
       </c>
       <c r="B24" s="22">
         <f>C23*B22*1000-C21</f>
-        <v/>
+        <v>56.530303030303045</v>
       </c>
     </row>
     <row r="25">
@@ -2545,11 +2542,11 @@
       </c>
       <c r="B25" s="23">
         <f>B24/AB_Inputs!$B$30</f>
-        <v/>
+        <v>48.73301985370953</v>
       </c>
       <c r="C25" s="22">
         <f>D13</f>
-        <v/>
+        <v>50.0</v>
       </c>
     </row>
     <row r="26">
@@ -2595,19 +2592,19 @@
       </c>
       <c r="C29" s="20">
         <f>AB_Inputs!$B$15</f>
-        <v/>
+        <v>150.0</v>
       </c>
       <c r="D29" s="20">
         <f>AB_Inputs!$B$19-AB_Inputs!$B$15</f>
-        <v/>
+        <v>208.0</v>
       </c>
       <c r="E29" s="20">
         <f>AB_Inputs!$B$22</f>
-        <v/>
+        <v>205.0</v>
       </c>
       <c r="F29" s="20">
         <f>AB_Inputs!$B$23</f>
-        <v/>
+        <v>205.0</v>
       </c>
     </row>
     <row r="30">
@@ -2625,14 +2622,14 @@
       </c>
       <c r="B31" s="27">
         <f>AB_Inputs!$B$33</f>
-        <v/>
+        <v>0.22</v>
       </c>
       <c r="C31" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D31" s="28">
         <f>13-AB_Inputs!$B$34</f>
-        <v/>
+        <v>11.0</v>
       </c>
       <c r="E31" s="12" t="n">
         <v>12</v>
@@ -2649,14 +2646,14 @@
       </c>
       <c r="B32" s="27">
         <f>AB_Inputs!$B$35</f>
-        <v/>
+        <v>0.13</v>
       </c>
       <c r="C32" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D32" s="28">
         <f>13-AB_Inputs!$B$36</f>
-        <v/>
+        <v>10.0</v>
       </c>
       <c r="E32" s="12" t="n">
         <v>12</v>
@@ -2673,14 +2670,14 @@
       </c>
       <c r="B33" s="27">
         <f>AB_Inputs!$B$37</f>
-        <v/>
+        <v>0.05</v>
       </c>
       <c r="C33" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D33" s="28">
         <f>13-AB_Inputs!$B$38</f>
-        <v/>
+        <v>4.0</v>
       </c>
       <c r="E33" s="12" t="n">
         <v>12</v>
@@ -2697,14 +2694,14 @@
       </c>
       <c r="B34" s="27">
         <f>AB_Inputs!$B$39</f>
-        <v/>
+        <v>0.26</v>
       </c>
       <c r="C34" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D34" s="28">
         <f>13-AB_Inputs!$B$40</f>
-        <v/>
+        <v>3.0</v>
       </c>
       <c r="E34" s="12" t="n">
         <v>12</v>
@@ -2721,14 +2718,14 @@
       </c>
       <c r="B35" s="27">
         <f>AB_Inputs!$B$41</f>
-        <v/>
+        <v>0.03</v>
       </c>
       <c r="C35" s="12" t="n">
         <v>0</v>
       </c>
       <c r="D35" s="28">
         <f>13-AB_Inputs!$B$42</f>
-        <v/>
+        <v>2.0</v>
       </c>
       <c r="E35" s="12" t="n">
         <v>12</v>
@@ -2745,7 +2742,7 @@
       </c>
       <c r="B36" s="29">
         <f>SUM(B31:B35)</f>
-        <v/>
+        <v>0.69</v>
       </c>
     </row>
     <row r="37">
@@ -2756,7 +2753,7 @@
       </c>
       <c r="B37" s="27">
         <f>AB_Inputs!$B$43</f>
-        <v/>
+        <v>0.75</v>
       </c>
     </row>
     <row r="38">
@@ -2767,19 +2764,19 @@
       </c>
       <c r="C38" s="21">
         <f>C29*SUMPRODUCT($B$31:$B$35,C31:C35)/12*$B$37</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="D38" s="21">
         <f>D29*SUMPRODUCT($B$31:$B$35,D31:D35)/12*$B$37</f>
-        <v/>
+        <v>61.879999999999995</v>
       </c>
       <c r="E38" s="21">
         <f>E29*SUMPRODUCT($B$31:$B$35,E31:E35)/12*$B$37</f>
-        <v/>
+        <v>106.0875</v>
       </c>
       <c r="F38" s="21">
         <f>F29*SUMPRODUCT($B$31:$B$35,F31:F35)/12*$B$37</f>
-        <v/>
+        <v>106.0875</v>
       </c>
     </row>
     <row r="39">
@@ -2791,19 +2788,19 @@
       <c r="B39" s="31" t="n"/>
       <c r="C39" s="32">
         <f>C29-C38</f>
-        <v/>
+        <v>150.0</v>
       </c>
       <c r="D39" s="32">
         <f>D29-D38</f>
-        <v/>
+        <v>146.12</v>
       </c>
       <c r="E39" s="32">
         <f>E29-E38</f>
-        <v/>
+        <v>98.9125</v>
       </c>
       <c r="F39" s="33">
         <f>IF(AB_Inputs!$B$44=1,F29*$B$36*(1-$B$37),F29-F38)</f>
-        <v/>
+        <v>98.9125</v>
       </c>
       <c r="G39" s="31" t="n"/>
     </row>
@@ -2856,15 +2853,15 @@
       </c>
       <c r="D43" s="27">
         <f>AB_Inputs!$B$48</f>
-        <v/>
+        <v>0.58</v>
       </c>
       <c r="E43" s="27">
         <f>AB_Inputs!$B$49</f>
-        <v/>
+        <v>0.43</v>
       </c>
       <c r="F43" s="27">
         <f>AB_Inputs!$B$50</f>
-        <v/>
+        <v>0.3</v>
       </c>
     </row>
     <row r="44">
@@ -2876,19 +2873,19 @@
       <c r="B44" s="31" t="n"/>
       <c r="C44" s="33">
         <f>AB_Inputs!$B$47</f>
-        <v/>
+        <v>190.0</v>
       </c>
       <c r="D44" s="32">
         <f>C44*(1+D43)</f>
-        <v/>
+        <v>300.2</v>
       </c>
       <c r="E44" s="32">
         <f>D44*(1+E43)</f>
-        <v/>
+        <v>429.28599999999994</v>
       </c>
       <c r="F44" s="32">
         <f>E44*(1+F43)</f>
-        <v/>
+        <v>558.0717999999999</v>
       </c>
       <c r="G44" s="31" t="n"/>
     </row>
@@ -2942,19 +2939,19 @@
       <c r="B48" s="31" t="n"/>
       <c r="C48" s="33">
         <f>AB_Inputs!$B$55</f>
-        <v/>
+        <v>5.0</v>
       </c>
       <c r="D48" s="33">
         <f>AB_Inputs!$B$56</f>
-        <v/>
+        <v>30.0</v>
       </c>
       <c r="E48" s="33">
         <f>AB_Inputs!$B$57</f>
-        <v/>
+        <v>75.0</v>
       </c>
       <c r="F48" s="33">
         <f>AB_Inputs!$B$58</f>
-        <v/>
+        <v>120.0</v>
       </c>
       <c r="G48" s="31" t="n"/>
     </row>
@@ -3007,19 +3004,19 @@
       </c>
       <c r="C52" s="21">
         <f>C39</f>
-        <v/>
+        <v>150.0</v>
       </c>
       <c r="D52" s="21">
         <f>D39</f>
-        <v/>
+        <v>146.12</v>
       </c>
       <c r="E52" s="21">
         <f>E39</f>
-        <v/>
+        <v>98.9125</v>
       </c>
       <c r="F52" s="21">
         <f>F39</f>
-        <v/>
+        <v>98.9125</v>
       </c>
     </row>
     <row r="53">
@@ -3030,19 +3027,19 @@
       </c>
       <c r="C53" s="21">
         <f>C48</f>
-        <v/>
+        <v>5.0</v>
       </c>
       <c r="D53" s="21">
         <f>D48</f>
-        <v/>
+        <v>30.0</v>
       </c>
       <c r="E53" s="21">
         <f>E48</f>
-        <v/>
+        <v>75.0</v>
       </c>
       <c r="F53" s="21">
         <f>F48</f>
-        <v/>
+        <v>120.0</v>
       </c>
     </row>
     <row r="54">
@@ -3053,19 +3050,19 @@
       </c>
       <c r="C54" s="21">
         <f>-C44</f>
-        <v/>
+        <v>-190.0</v>
       </c>
       <c r="D54" s="21">
         <f>-D44</f>
-        <v/>
+        <v>-300.2</v>
       </c>
       <c r="E54" s="21">
         <f>-E44</f>
-        <v/>
+        <v>-429.28599999999994</v>
       </c>
       <c r="F54" s="21">
         <f>-F44</f>
-        <v/>
+        <v>-558.0717999999999</v>
       </c>
     </row>
     <row r="55">
@@ -3076,19 +3073,19 @@
       </c>
       <c r="C55" s="21">
         <f>C52+C53+C54</f>
-        <v/>
+        <v>-35.0</v>
       </c>
       <c r="D55" s="21">
         <f>D52+D53+D54</f>
-        <v/>
+        <v>-124.07999999999998</v>
       </c>
       <c r="E55" s="21">
         <f>E52+E53+E54</f>
-        <v/>
+        <v>-255.37349999999995</v>
       </c>
       <c r="F55" s="21">
         <f>F52+F53+F54</f>
-        <v/>
+        <v>-339.1592999999999</v>
       </c>
     </row>
     <row r="56">
@@ -3099,19 +3096,19 @@
       </c>
       <c r="C56" s="20">
         <f>AB_Inputs!$B$6</f>
-        <v/>
+        <v>15673.0</v>
       </c>
       <c r="D56" s="20">
         <f>AB_Inputs!$B$7</f>
-        <v/>
+        <v>17186.0</v>
       </c>
       <c r="E56" s="20">
         <f>AB_Inputs!$B$8</f>
-        <v/>
+        <v>19500.0</v>
       </c>
       <c r="F56" s="20">
         <f>AB_Inputs!$B$9</f>
-        <v/>
+        <v>21300.0</v>
       </c>
     </row>
     <row r="57">
@@ -3164,19 +3161,19 @@
       <c r="B60" s="31" t="n"/>
       <c r="C60" s="32">
         <f>C55</f>
-        <v/>
+        <v>-35.0</v>
       </c>
       <c r="D60" s="32">
         <f>D55</f>
-        <v/>
+        <v>-124.07999999999998</v>
       </c>
       <c r="E60" s="32">
         <f>E55</f>
-        <v/>
+        <v>-255.37349999999995</v>
       </c>
       <c r="F60" s="32">
         <f>F55</f>
-        <v/>
+        <v>-339.1592999999999</v>
       </c>
       <c r="G60" s="31" t="n"/>
     </row>
@@ -3189,19 +3186,19 @@
       <c r="B61" s="31" t="n"/>
       <c r="C61" s="34">
         <f>C55/C56*10000</f>
-        <v/>
+        <v>-22.331397945511387</v>
       </c>
       <c r="D61" s="34">
         <f>D55/D56*10000</f>
-        <v/>
+        <v>-72.19830094262771</v>
       </c>
       <c r="E61" s="34">
         <f>E55/E56*10000</f>
-        <v/>
+        <v>-130.96076923076922</v>
       </c>
       <c r="F61" s="34">
         <f>F55/F56*10000</f>
-        <v/>
+        <v>-159.22971830985912</v>
       </c>
       <c r="G61" s="31" t="n"/>
     </row>
@@ -3215,15 +3212,15 @@
       <c r="C62" s="31" t="n"/>
       <c r="D62" s="32">
         <f>D55-C55</f>
-        <v/>
+        <v>-89.07999999999998</v>
       </c>
       <c r="E62" s="32">
         <f>E55-D55</f>
-        <v/>
+        <v>-131.29349999999997</v>
       </c>
       <c r="F62" s="32">
         <f>F55-E55</f>
-        <v/>
+        <v>-83.78579999999997</v>
       </c>
       <c r="G62" s="31" t="n"/>
     </row>
@@ -3237,15 +3234,15 @@
       <c r="C63" s="31" t="n"/>
       <c r="D63" s="34">
         <f>D62/D56*10000</f>
-        <v/>
+        <v>-51.832887233794935</v>
       </c>
       <c r="E63" s="34">
         <f>E62/E56*10000</f>
-        <v/>
+        <v>-67.32999999999998</v>
       </c>
       <c r="F63" s="34">
         <f>F62/F56*10000</f>
-        <v/>
+        <v>-39.33605633802816</v>
       </c>
       <c r="G63" s="31" t="n"/>
     </row>
@@ -3257,15 +3254,15 @@
       </c>
       <c r="D64" s="21">
         <f>D52-C52</f>
-        <v/>
+        <v>-3.8799999999999955</v>
       </c>
       <c r="E64" s="21">
         <f>E52-D52</f>
-        <v/>
+        <v>-47.20750000000001</v>
       </c>
       <c r="F64" s="21">
         <f>F52-E52</f>
-        <v/>
+        <v>0.0</v>
       </c>
     </row>
     <row r="65">
@@ -3276,15 +3273,15 @@
       </c>
       <c r="D65" s="21">
         <f>D54-C54</f>
-        <v/>
+        <v>-110.19999999999999</v>
       </c>
       <c r="E65" s="21">
         <f>E54-D54</f>
-        <v/>
+        <v>-129.08599999999996</v>
       </c>
       <c r="F65" s="21">
         <f>F54-E54</f>
-        <v/>
+        <v>-128.7858</v>
       </c>
     </row>
     <row r="66">
@@ -3295,15 +3292,15 @@
       </c>
       <c r="D66" s="21">
         <f>D53-C53</f>
-        <v/>
+        <v>25.0</v>
       </c>
       <c r="E66" s="21">
         <f>E53-D53</f>
-        <v/>
+        <v>45.0</v>
       </c>
       <c r="F66" s="21">
         <f>F53-E53</f>
-        <v/>
+        <v>45.0</v>
       </c>
     </row>
     <row r="67">
@@ -3314,11 +3311,11 @@
       </c>
       <c r="E67" s="35">
         <f>AB_Inputs!$B$61</f>
-        <v/>
+        <v>115.0</v>
       </c>
       <c r="F67" s="35">
         <f>AB_Inputs!$B$62</f>
-        <v/>
+        <v>130.0</v>
       </c>
     </row>
     <row r="68">
@@ -3329,11 +3326,11 @@
       </c>
       <c r="E68" s="29">
         <f>-E63/E67</f>
-        <v/>
+        <v>0.5854782608695651</v>
       </c>
       <c r="F68" s="29">
         <f>-F63/F67</f>
-        <v/>
+        <v>0.3025850487540627</v>
       </c>
     </row>
     <row r="69">
@@ -3344,7 +3341,7 @@
       </c>
       <c r="C69" s="20">
         <f>AB_Inputs!$B$65</f>
-        <v/>
+        <v>500.0</v>
       </c>
     </row>
     <row r="70">
@@ -3365,30 +3362,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Audiobooks: sensitivity on licensing-cost growth</t>
+          <t>Audiobooks: sensitivity to the growth assigned to audiobook licensing cost</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B, A and group revenue are held at the AB_Bridge values; only C moves. Headwind = y/y change in N as bp of group revenue (negative = margin drag). Blue cells are the scenario values and can be edited.</t>
+          <t>Only C moves. B, A and group revenue are held at the AB_Bridge values. The row's growth rate is applied to both 2026E and 2027E; 2025 growth stays at the inputs value. Blue cells can be edited.</t>
         </is>
       </c>
     </row>
@@ -3396,639 +3392,291 @@
       <c r="A3" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>Table 1. Cost growth p.a. applied to both 2026E and 2027E (base case on AB_Inputs: 43% then 30%)</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="n"/>
-      <c r="C4" s="4" t="n"/>
-      <c r="D4" s="4" t="n"/>
-      <c r="E4" s="4" t="n"/>
-      <c r="F4" s="4" t="n"/>
-      <c r="G4" s="4" t="n"/>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Licensing-cost growth p.a., 2026E and 2027E</t>
+        </is>
+      </c>
+      <c r="B4" s="36" t="inlineStr">
+        <is>
+          <t>C 2026E, €M</t>
+        </is>
+      </c>
+      <c r="C4" s="36" t="inlineStr">
+        <is>
+          <t>C 2027E, €M</t>
+        </is>
+      </c>
+      <c r="D4" s="36" t="inlineStr">
+        <is>
+          <t>Contribution 2026E, €M</t>
+        </is>
+      </c>
+      <c r="E4" s="36" t="inlineStr">
+        <is>
+          <t>Contribution 2027E, €M</t>
+        </is>
+      </c>
+      <c r="F4" s="36" t="inlineStr">
+        <is>
+          <t>Headwind 2026E, bp</t>
+        </is>
+      </c>
+      <c r="G4" s="36" t="inlineStr">
+        <is>
+          <t>Headwind 2027E, bp</t>
+        </is>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="18" t="inlineStr">
-        <is>
-          <t>Cost growth p.a.</t>
-        </is>
-      </c>
-      <c r="B5" s="19" t="inlineStr">
-        <is>
-          <t>C 2026E</t>
-        </is>
-      </c>
-      <c r="C5" s="19" t="inlineStr">
-        <is>
-          <t>C 2027E</t>
-        </is>
-      </c>
-      <c r="D5" s="19" t="inlineStr">
-        <is>
-          <t>N 2026E</t>
-        </is>
-      </c>
-      <c r="E5" s="19" t="inlineStr">
-        <is>
-          <t>N 2027E</t>
-        </is>
-      </c>
-      <c r="F5" s="19" t="inlineStr">
-        <is>
-          <t>Headwind 2026E, bp</t>
-        </is>
-      </c>
-      <c r="G5" s="19" t="inlineStr">
-        <is>
-          <t>Headwind 2027E, bp</t>
-        </is>
-      </c>
-      <c r="H5" s="19" t="inlineStr">
-        <is>
-          <t>Share of consensus 2026E</t>
-        </is>
+      <c r="A5" s="37" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="B5" s="20">
+        <f>AB_Bridge!$D$44*(1+$A5)</f>
+        <v>360.23999999999995</v>
+      </c>
+      <c r="C5" s="20">
+        <f>AB_Bridge!$D$44*(1+$A5)^2</f>
+        <v>432.28799999999995</v>
+      </c>
+      <c r="D5" s="20">
+        <f>AB_Bridge!$E$39+AB_Bridge!$E$48-B5</f>
+        <v>-186.32749999999996</v>
+      </c>
+      <c r="E5" s="20">
+        <f>AB_Bridge!$F$39+AB_Bridge!$F$48-C5</f>
+        <v>-213.37549999999996</v>
+      </c>
+      <c r="F5" s="35">
+        <f>(D5-AB_Bridge!$D$55)/AB_Bridge!$E$56*10000</f>
+        <v>-31.92179487179486</v>
+      </c>
+      <c r="G5" s="35">
+        <f>(E5-D5)/AB_Bridge!$F$56*10000</f>
+        <v>-12.698591549295775</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="36" t="n">
-        <v>0.2</v>
+      <c r="A6" s="37" t="n">
+        <v>0.3</v>
       </c>
       <c r="B6" s="20">
         <f>AB_Bridge!$D$44*(1+$A6)</f>
-        <v/>
+        <v>390.26</v>
       </c>
       <c r="C6" s="20">
         <f>AB_Bridge!$D$44*(1+$A6)^2</f>
-        <v/>
+        <v>507.338</v>
       </c>
       <c r="D6" s="20">
         <f>AB_Bridge!$E$39+AB_Bridge!$E$48-B6</f>
-        <v/>
+        <v>-216.3475</v>
       </c>
       <c r="E6" s="20">
         <f>AB_Bridge!$F$39+AB_Bridge!$F$48-C6</f>
-        <v/>
+        <v>-288.42550000000006</v>
       </c>
       <c r="F6" s="35">
         <f>(D6-AB_Bridge!$D$55)/AB_Bridge!$E$56*10000</f>
-        <v/>
+        <v>-47.31666666666667</v>
       </c>
       <c r="G6" s="35">
         <f>(E6-D6)/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="H6" s="27">
-        <f>-F6/AB_Bridge!$E$67</f>
-        <v/>
+        <v>-33.839436619718334</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="36" t="n">
-        <v>0.3</v>
+      <c r="A7" s="37" t="n">
+        <v>0.4</v>
       </c>
       <c r="B7" s="20">
         <f>AB_Bridge!$D$44*(1+$A7)</f>
-        <v/>
+        <v>420.28</v>
       </c>
       <c r="C7" s="20">
         <f>AB_Bridge!$D$44*(1+$A7)^2</f>
-        <v/>
+        <v>588.3919999999999</v>
       </c>
       <c r="D7" s="20">
         <f>AB_Bridge!$E$39+AB_Bridge!$E$48-B7</f>
-        <v/>
+        <v>-246.36749999999998</v>
       </c>
       <c r="E7" s="20">
         <f>AB_Bridge!$F$39+AB_Bridge!$F$48-C7</f>
-        <v/>
+        <v>-369.4794999999999</v>
       </c>
       <c r="F7" s="35">
         <f>(D7-AB_Bridge!$D$55)/AB_Bridge!$E$56*10000</f>
-        <v/>
+        <v>-62.71153846153845</v>
       </c>
       <c r="G7" s="35">
         <f>(E7-D7)/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="H7" s="27">
-        <f>-F7/AB_Bridge!$E$67</f>
-        <v/>
+        <v>-57.79906103286382</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="36" t="n">
-        <v>0.4</v>
+      <c r="A8" s="37" t="n">
+        <v>0.43</v>
       </c>
       <c r="B8" s="20">
         <f>AB_Bridge!$D$44*(1+$A8)</f>
-        <v/>
+        <v>429.28599999999994</v>
       </c>
       <c r="C8" s="20">
         <f>AB_Bridge!$D$44*(1+$A8)^2</f>
-        <v/>
+        <v>613.8789799999998</v>
       </c>
       <c r="D8" s="20">
         <f>AB_Bridge!$E$39+AB_Bridge!$E$48-B8</f>
-        <v/>
+        <v>-255.37349999999995</v>
       </c>
       <c r="E8" s="20">
         <f>AB_Bridge!$F$39+AB_Bridge!$F$48-C8</f>
-        <v/>
+        <v>-394.9664799999998</v>
       </c>
       <c r="F8" s="35">
         <f>(D8-AB_Bridge!$D$55)/AB_Bridge!$E$56*10000</f>
-        <v/>
+        <v>-67.32999999999998</v>
       </c>
       <c r="G8" s="35">
         <f>(E8-D8)/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="H8" s="27">
-        <f>-F8/AB_Bridge!$E$67</f>
-        <v/>
+        <v>-65.53661032863843</v>
+      </c>
+      <c r="H8" s="38" t="inlineStr">
+        <is>
+          <t>base 2026E growth</t>
+        </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="36" t="n">
-        <v>0.43</v>
+      <c r="A9" s="37" t="n">
+        <v>0.5</v>
       </c>
       <c r="B9" s="20">
         <f>AB_Bridge!$D$44*(1+$A9)</f>
-        <v/>
+        <v>450.29999999999995</v>
       </c>
       <c r="C9" s="20">
         <f>AB_Bridge!$D$44*(1+$A9)^2</f>
-        <v/>
+        <v>675.4499999999999</v>
       </c>
       <c r="D9" s="20">
         <f>AB_Bridge!$E$39+AB_Bridge!$E$48-B9</f>
-        <v/>
+        <v>-276.38749999999993</v>
       </c>
       <c r="E9" s="20">
         <f>AB_Bridge!$F$39+AB_Bridge!$F$48-C9</f>
-        <v/>
+        <v>-456.5374999999999</v>
       </c>
       <c r="F9" s="35">
         <f>(D9-AB_Bridge!$D$55)/AB_Bridge!$E$56*10000</f>
-        <v/>
+        <v>-78.10641025641023</v>
       </c>
       <c r="G9" s="35">
         <f>(E9-D9)/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="H9" s="27">
-        <f>-F9/AB_Bridge!$E$67</f>
-        <v/>
-      </c>
-      <c r="I9" s="37" t="inlineStr">
-        <is>
-          <t>base 2026E growth</t>
-        </is>
+        <v>-84.57746478873239</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="36" t="n">
-        <v>0.5</v>
+      <c r="A10" s="37" t="n">
+        <v>0.6</v>
       </c>
       <c r="B10" s="20">
         <f>AB_Bridge!$D$44*(1+$A10)</f>
-        <v/>
+        <v>480.32</v>
       </c>
       <c r="C10" s="20">
         <f>AB_Bridge!$D$44*(1+$A10)^2</f>
-        <v/>
+        <v>768.5120000000002</v>
       </c>
       <c r="D10" s="20">
         <f>AB_Bridge!$E$39+AB_Bridge!$E$48-B10</f>
-        <v/>
+        <v>-306.4075</v>
       </c>
       <c r="E10" s="20">
         <f>AB_Bridge!$F$39+AB_Bridge!$F$48-C10</f>
-        <v/>
+        <v>-549.5995000000001</v>
       </c>
       <c r="F10" s="35">
         <f>(D10-AB_Bridge!$D$55)/AB_Bridge!$E$56*10000</f>
-        <v/>
+        <v>-93.50128205128208</v>
       </c>
       <c r="G10" s="35">
         <f>(E10-D10)/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="H10" s="27">
-        <f>-F10/AB_Bridge!$E$67</f>
-        <v/>
+        <v>-114.174647887324</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="36" t="n">
-        <v>0.6</v>
+      <c r="A11" s="37" t="n">
+        <v>0.7</v>
       </c>
       <c r="B11" s="20">
         <f>AB_Bridge!$D$44*(1+$A11)</f>
-        <v/>
+        <v>510.34</v>
       </c>
       <c r="C11" s="20">
         <f>AB_Bridge!$D$44*(1+$A11)^2</f>
-        <v/>
+        <v>867.5779999999999</v>
       </c>
       <c r="D11" s="20">
         <f>AB_Bridge!$E$39+AB_Bridge!$E$48-B11</f>
-        <v/>
+        <v>-336.4275</v>
       </c>
       <c r="E11" s="20">
         <f>AB_Bridge!$F$39+AB_Bridge!$F$48-C11</f>
-        <v/>
+        <v>-648.6654999999998</v>
       </c>
       <c r="F11" s="35">
         <f>(D11-AB_Bridge!$D$55)/AB_Bridge!$E$56*10000</f>
-        <v/>
+        <v>-108.89615384615387</v>
       </c>
       <c r="G11" s="35">
         <f>(E11-D11)/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="H11" s="27">
-        <f>-F11/AB_Bridge!$E$67</f>
-        <v/>
+        <v>-146.5906103286384</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="36" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="B12" s="20">
-        <f>AB_Bridge!$D$44*(1+$A12)</f>
-        <v/>
-      </c>
-      <c r="C12" s="20">
-        <f>AB_Bridge!$D$44*(1+$A12)^2</f>
-        <v/>
-      </c>
-      <c r="D12" s="20">
-        <f>AB_Bridge!$E$39+AB_Bridge!$E$48-B12</f>
-        <v/>
-      </c>
-      <c r="E12" s="20">
-        <f>AB_Bridge!$F$39+AB_Bridge!$F$48-C12</f>
-        <v/>
-      </c>
-      <c r="F12" s="35">
-        <f>(D12-AB_Bridge!$D$55)/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="G12" s="35">
-        <f>(E12-D12)/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="H12" s="27">
-        <f>-F12/AB_Bridge!$E$67</f>
-        <v/>
-      </c>
+      <c r="A12" t="inlineStr"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
+      <c r="A13" s="30" t="inlineStr">
+        <is>
+          <t>Base case on AB_Bridge (43% in 2026E, 30% in 2027E)</t>
+        </is>
+      </c>
+      <c r="B13" s="33">
+        <f>AB_Bridge!$E$44</f>
+        <v>429.28599999999994</v>
+      </c>
+      <c r="C13" s="33">
+        <f>AB_Bridge!$F$44</f>
+        <v>558.0717999999999</v>
+      </c>
+      <c r="D13" s="33">
+        <f>AB_Bridge!$E$55</f>
+        <v>-255.37349999999995</v>
+      </c>
+      <c r="E13" s="33">
+        <f>AB_Bridge!$F$55</f>
+        <v>-339.1592999999999</v>
+      </c>
+      <c r="F13" s="39">
+        <f>AB_Bridge!$E$63</f>
+        <v>-67.32999999999998</v>
+      </c>
+      <c r="G13" s="39">
+        <f>AB_Bridge!$F$63</f>
+        <v>-39.33605633802816</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Table 2. Headwind 2026E (bp) by 2024 cost anchor (rows, €M) and 2026E cost growth (columns); 2025 growth held at the AB_Inputs value</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="n"/>
-      <c r="C14" s="4" t="n"/>
-      <c r="D14" s="4" t="n"/>
-      <c r="E14" s="4" t="n"/>
-      <c r="F14" s="4" t="n"/>
-      <c r="G14" s="4" t="n"/>
+      <c r="A14" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="18" t="inlineStr">
-        <is>
-          <t>2024 anchor, €M  \  2026E growth</t>
-        </is>
-      </c>
-      <c r="B15" s="38" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C15" s="38" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="D15" s="38" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="E15" s="38" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F15" s="38" t="n">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="5" t="n">
-        <v>150</v>
-      </c>
-      <c r="B16" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A16*(1+AB_Inputs!$B$48)*(1+B$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A16*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="C16" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A16*(1+AB_Inputs!$B$48)*(1+C$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A16*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="D16" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A16*(1+AB_Inputs!$B$48)*(1+D$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A16*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="E16" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A16*(1+AB_Inputs!$B$48)*(1+E$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A16*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="F16" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A16*(1+AB_Inputs!$B$48)*(1+F$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A16*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="5" t="n">
-        <v>190</v>
-      </c>
-      <c r="B17" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A17*(1+AB_Inputs!$B$48)*(1+B$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A17*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="C17" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A17*(1+AB_Inputs!$B$48)*(1+C$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A17*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="D17" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A17*(1+AB_Inputs!$B$48)*(1+D$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A17*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="E17" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A17*(1+AB_Inputs!$B$48)*(1+E$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A17*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="F17" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A17*(1+AB_Inputs!$B$48)*(1+F$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A17*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="H17" s="37" t="inlineStr">
-        <is>
-          <t>base anchor</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="n">
-        <v>250</v>
-      </c>
-      <c r="B18" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A18*(1+AB_Inputs!$B$48)*(1+B$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A18*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="C18" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A18*(1+AB_Inputs!$B$48)*(1+C$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A18*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="D18" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A18*(1+AB_Inputs!$B$48)*(1+D$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A18*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="E18" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A18*(1+AB_Inputs!$B$48)*(1+E$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A18*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="F18" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A18*(1+AB_Inputs!$B$48)*(1+F$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A18*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="5" t="n">
-        <v>300</v>
-      </c>
-      <c r="B19" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A19*(1+AB_Inputs!$B$48)*(1+B$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A19*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="C19" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A19*(1+AB_Inputs!$B$48)*(1+C$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A19*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="D19" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A19*(1+AB_Inputs!$B$48)*(1+D$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A19*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="E19" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A19*(1+AB_Inputs!$B$48)*(1+E$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A19*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="F19" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A19*(1+AB_Inputs!$B$48)*(1+F$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A19*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="5" t="n">
-        <v>350</v>
-      </c>
-      <c r="B20" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A20*(1+AB_Inputs!$B$48)*(1+B$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A20*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="C20" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A20*(1+AB_Inputs!$B$48)*(1+C$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A20*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="D20" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A20*(1+AB_Inputs!$B$48)*(1+D$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A20*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="E20" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A20*(1+AB_Inputs!$B$48)*(1+E$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A20*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-      <c r="F20" s="35">
-        <f>((AB_Bridge!$E$39+AB_Bridge!$E$48-$A20*(1+AB_Inputs!$B$48)*(1+F$15))-(AB_Bridge!$D$39+AB_Bridge!$D$48-$A20*(1+AB_Inputs!$B$48)))/AB_Bridge!$E$56*10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>Table 3. Headwind 2027E (bp) by 2026E cost growth (rows) and 2027E cost growth (columns)</t>
-        </is>
-      </c>
-      <c r="B22" s="4" t="n"/>
-      <c r="C22" s="4" t="n"/>
-      <c r="D22" s="4" t="n"/>
-      <c r="E22" s="4" t="n"/>
-      <c r="F22" s="4" t="n"/>
-      <c r="G22" s="4" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="18" t="inlineStr">
-        <is>
-          <t>2026E growth  \  2027E growth</t>
-        </is>
-      </c>
-      <c r="B23" s="38" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="C23" s="38" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="D23" s="38" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="E23" s="38" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F23" s="38" t="n">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="36" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="B24" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A24)*(1+B$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A24)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="C24" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A24)*(1+C$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A24)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="D24" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A24)*(1+D$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A24)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="E24" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A24)*(1+E$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A24)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="F24" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A24)*(1+F$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A24)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="36" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="B25" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A25)*(1+B$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A25)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="C25" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A25)*(1+C$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A25)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="D25" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A25)*(1+D$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A25)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="E25" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A25)*(1+E$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A25)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="F25" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A25)*(1+F$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A25)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="36" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="B26" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A26)*(1+B$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A26)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="C26" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A26)*(1+C$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A26)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="D26" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A26)*(1+D$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A26)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="E26" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A26)*(1+E$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A26)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="F26" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A26)*(1+F$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A26)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="H26" s="37" t="inlineStr">
-        <is>
-          <t>base 2026E growth; base 2027E growth is 30%</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="36" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="B27" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A27)*(1+B$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A27)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="C27" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A27)*(1+C$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A27)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="D27" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A27)*(1+D$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A27)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="E27" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A27)*(1+E$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A27)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="F27" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A27)*(1+F$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A27)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="36" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="B28" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A28)*(1+B$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A28)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="C28" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A28)*(1+C$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A28)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="D28" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A28)*(1+D$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A28)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="E28" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A28)*(1+E$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A28)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-      <c r="F28" s="35">
-        <f>((AB_Bridge!$F$39+AB_Bridge!$F$48-AB_Bridge!$D$44*(1+$A28)*(1+F$23))-(AB_Bridge!$E$39+AB_Bridge!$E$48-AB_Bridge!$D$44*(1+$A28)))/AB_Bridge!$F$56*10000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr"/>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>Reading: the headwind stays negative in every cell except the 10% column of Table 3, where paid revenue growth of about €45M outruns a 10% rise in cost. The size is driven by the cost growth assumption. The 2026E headwind rests on listeners +60% (disclosed) and the 0.7x haircut from listeners to cost (estimate).</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Reading: the headwind is negative in every row. Its size scales with the growth assigned to licensing cost, which rests on listeners +60% (disclosed) and a 0.7x haircut from listeners to cost (estimate).</t>
         </is>
       </c>
     </row>

</xml_diff>